<commit_message>
U2TC: las tablas usan las fórmulas del ejemplo de la profesora
nqx = 2·n·nmx/(2+n·nmx), nAx = 0.12, 1.5 y 2.5 (1/nmx en el grupo abierto), lx+n = lx·npx y ndx = lx·nqx, con el orden de columnas del ejemplo (sin nZx). Se quita Coale-Demeny. Se actualizan el cálculo de referencia, la verificación y el README.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qxava2B1gmXGAGJzmKd5vp
</commit_message>
<xml_diff>
--- a/tablas-de-mortalidad/tarea-inegi-tablas-transversales/resultados/Fuentes_de_consulta.xlsx
+++ b/tablas-de-mortalidad/tarea-inegi-tablas-transversales/resultados/Fuentes_de_consulta.xlsx
@@ -441,7 +441,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -548,19 +548,15 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="14" fillId="6" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="14" fillId="6" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="9" fillId="6" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="14" fillId="10" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="14" fillId="10" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="14" fillId="10" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="14" fillId="10" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="9" fillId="10" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="14" fillId="6" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="14" fillId="10" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="10" fillId="8" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
@@ -697,7 +693,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Tabla hombres'!$K$9:$K$25</f>
+              <f>'Tabla hombres'!$J$9:$J$25</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -738,7 +734,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Tabla mujeres'!$K$9:$K$25</f>
+              <f>'Tabla mujeres'!$J$9:$J$25</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -779,7 +775,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Tabla ambos sexos'!$K$9:$K$25</f>
+              <f>'Tabla ambos sexos'!$J$9:$J$25</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1120,7 +1116,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Tabla hombres'!$I$9:$I$24</f>
+              <f>'Tabla hombres'!$H$9:$H$24</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1161,7 +1157,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Tabla mujeres'!$I$9:$I$24</f>
+              <f>'Tabla mujeres'!$H$9:$H$24</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1202,7 +1198,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Tabla ambos sexos'!$I$9:$I$24</f>
+              <f>'Tabla ambos sexos'!$H$9:$H$24</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -5543,11 +5539,11 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="9" customWidth="1" min="15" max="15"/>
@@ -5663,7 +5659,7 @@
       <c r="A6" s="29" t="n"/>
       <c r="B6" s="35" t="inlineStr">
         <is>
-          <t>nMx = D/P;  nqx = n·nMx / (1 + (n − nax)·nMx);  lx+n = lx·(1 − nqx);  ndx = lx − lx+n;  nLx = n·lx+n + nax·ndx;  Tx = suma de nLx hacia abajo;  ex = Tx/lx.  Grupo abierto 75+: q = 1 y L = l/M.</t>
+          <t>nmx = D/P;  nqx = (2·n·nmx) / (2 + n·nmx);  npx = 1 − nqx;  lx+n = lx·npx;  ndx = lx·nqx;  nLx = lx+n·n + ndx·nAx;  Tx = suma de nLx hacia abajo;  ex = Tx/lx.</t>
         </is>
       </c>
       <c r="P6" s="29" t="n"/>
@@ -5672,7 +5668,7 @@
       <c r="A7" s="29" t="n"/>
       <c r="B7" s="35" t="inlineStr">
         <is>
-          <t>nax: para 0 y 1-4, Coale-Demeny según la mortalidad infantil y el sexo (en ambos sexos, el promedio de hombres y mujeres); n/2 en los demás grupos. Valores sin redondear.</t>
+          <t>nAx: 0.12 en la edad 0, 1.5 en 1-4 y 2.5 en los demás grupos (los valores del Cuadro 4.3 del ejemplo de la profesora). En el grupo abierto 75+: nqx = 1 y nAx = 1/nmx.</t>
         </is>
       </c>
       <c r="P7" s="29" t="n"/>
@@ -5706,32 +5702,32 @@
       </c>
       <c r="G8" s="37" t="inlineStr">
         <is>
-          <t>nMx</t>
+          <t>nmx</t>
         </is>
       </c>
       <c r="H8" s="37" t="inlineStr">
         <is>
-          <t>nax</t>
+          <t>nqx</t>
         </is>
       </c>
       <c r="I8" s="37" t="inlineStr">
         <is>
-          <t>nqx</t>
+          <t>npx</t>
         </is>
       </c>
       <c r="J8" s="37" t="inlineStr">
         <is>
-          <t>npx</t>
+          <t>lx</t>
         </is>
       </c>
       <c r="K8" s="37" t="inlineStr">
         <is>
-          <t>lx</t>
+          <t>ndx</t>
         </is>
       </c>
       <c r="L8" s="37" t="inlineStr">
         <is>
-          <t>ndx</t>
+          <t>nAx</t>
         </is>
       </c>
       <c r="M8" s="37" t="inlineStr">
@@ -5775,37 +5771,36 @@
         <f>F9/E9</f>
         <v>0.0100217282703059</v>
       </c>
-      <c r="H9" s="50">
-        <f>IF($G$9&gt;=0.107,0.33,0.045+2.684*$G$9)</f>
-        <v>0.071898318677501</v>
+      <c r="H9" s="55">
+        <f>(2*D9*G9)/(2+D9*G9)</f>
+        <v>0.00997176113009477</v>
       </c>
       <c r="I9" s="55">
-        <f>D9*G9/(1+(D9-H9)*G9)</f>
-        <v>0.00992937335308912</v>
-      </c>
-      <c r="J9" s="55">
-        <f>1-I9</f>
-        <v>0.990070626646911</v>
-      </c>
-      <c r="K9" s="39">
+        <f>1-H9</f>
+        <v>0.990028238869905</v>
+      </c>
+      <c r="J9" s="39">
         <f>$D$5</f>
         <v>100000</v>
       </c>
-      <c r="L9" s="39">
-        <f>K9*I9</f>
-        <v>992.937335308912</v>
+      <c r="K9" s="39">
+        <f>J9*H9</f>
+        <v>997.176113009477</v>
+      </c>
+      <c r="L9" s="56" t="n">
+        <v>0.12</v>
       </c>
       <c r="M9" s="39">
-        <f>D9*K10+H9*L9</f>
-        <v>99078.4531896519</v>
+        <f>J10*D9+K9*L9</f>
+        <v>99122.4850205517</v>
       </c>
       <c r="N9" s="39">
         <f>SUM(M9:$M$25)</f>
-        <v>7664264.49219202</v>
-      </c>
-      <c r="O9" s="56">
-        <f>N9/K9</f>
-        <v>76.6426449219202</v>
+        <v>7663958.31777888</v>
+      </c>
+      <c r="O9" s="57">
+        <f>N9/J9</f>
+        <v>76.6395831777888</v>
       </c>
       <c r="P9" s="29" t="n"/>
     </row>
@@ -5815,10 +5810,10 @@
         <f>'Cohorte ficticio'!B49</f>
         <v>1-4</v>
       </c>
-      <c r="C10" s="57" t="n">
+      <c r="C10" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="58" t="n">
+      <c r="D10" s="59" t="n">
         <v>4</v>
       </c>
       <c r="E10" s="42">
@@ -5833,37 +5828,36 @@
         <f>F10/E10</f>
         <v>0.000487233357771751</v>
       </c>
-      <c r="H10" s="59">
-        <f>IF($G$9&gt;=0.107,1.352,1.651-2.816*$G$9)</f>
-        <v>1.62277881319082</v>
+      <c r="H10" s="49">
+        <f>(2*D10*G10)/(2+D10*G10)</f>
+        <v>0.00194703610920462</v>
       </c>
       <c r="I10" s="49">
-        <f>D10*G10/(1+(D10-H10)*G10)</f>
-        <v>0.00194667866820864</v>
-      </c>
-      <c r="J10" s="49">
-        <f>1-I10</f>
-        <v>0.998053321331791</v>
+        <f>1-H10</f>
+        <v>0.998052963890795</v>
+      </c>
+      <c r="J10" s="42">
+        <f>J9*I9</f>
+        <v>99002.8238869905</v>
       </c>
       <c r="K10" s="42">
-        <f>K9-L9</f>
-        <v>99007.0626646911</v>
-      </c>
-      <c r="L10" s="42">
-        <f>K10*I10</f>
-        <v>192.73493689135</v>
+        <f>J10*H10</f>
+        <v>192.762073021196</v>
+      </c>
+      <c r="L10" s="60" t="n">
+        <v>1.5</v>
       </c>
       <c r="M10" s="42">
-        <f>D10*K11+H10*L10</f>
-        <v>395570.077083348</v>
+        <f>J11*D10+K10*L10</f>
+        <v>395529.390365409</v>
       </c>
       <c r="N10" s="42">
         <f>SUM(M10:$M$25)</f>
-        <v>7565186.03900237</v>
-      </c>
-      <c r="O10" s="60">
-        <f>N10/K10</f>
-        <v>76.4105694623374</v>
+        <v>7564835.83275833</v>
+      </c>
+      <c r="O10" s="61">
+        <f>N10/J10</f>
+        <v>76.4103036231917</v>
       </c>
       <c r="P10" s="29" t="n"/>
     </row>
@@ -5891,36 +5885,35 @@
         <f>F11/E11</f>
         <v>0.000224456677469159</v>
       </c>
-      <c r="H11" s="50">
-        <f>D11/2</f>
+      <c r="H11" s="55">
+        <f>(2*D11*G11)/(2+D11*G11)</f>
+        <v>0.00112165398053145</v>
+      </c>
+      <c r="I11" s="55">
+        <f>1-H11</f>
+        <v>0.998878346019469</v>
+      </c>
+      <c r="J11" s="39">
+        <f>J10*I10</f>
+        <v>98810.0618139693</v>
+      </c>
+      <c r="K11" s="39">
+        <f>J11*H11</f>
+        <v>110.830699150197</v>
+      </c>
+      <c r="L11" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I11" s="55">
-        <f>D11*G11/(1+(D11-H11)*G11)</f>
-        <v>0.00112165398053145</v>
-      </c>
-      <c r="J11" s="55">
-        <f>1-I11</f>
-        <v>0.998878346019469</v>
-      </c>
-      <c r="K11" s="39">
-        <f>K10-L10</f>
-        <v>98814.3277277997</v>
-      </c>
-      <c r="L11" s="39">
-        <f>K11*I11</f>
-        <v>110.835484029425</v>
-      </c>
       <c r="M11" s="39">
-        <f>D11*K12+H11*L11</f>
-        <v>493794.549928925</v>
+        <f>J12*D11+K11*L11</f>
+        <v>493773.232321971</v>
       </c>
       <c r="N11" s="39">
         <f>SUM(M11:$M$25)</f>
-        <v>7169615.96191902</v>
-      </c>
-      <c r="O11" s="56">
-        <f>N11/K11</f>
+        <v>7169306.44239292</v>
+      </c>
+      <c r="O11" s="57">
+        <f>N11/J11</f>
         <v>72.5564412244842</v>
       </c>
       <c r="P11" s="29" t="n"/>
@@ -5931,10 +5924,10 @@
         <f>'Cohorte ficticio'!B51</f>
         <v>10-14</v>
       </c>
-      <c r="C12" s="57" t="n">
+      <c r="C12" s="58" t="n">
         <v>10</v>
       </c>
-      <c r="D12" s="58" t="n">
+      <c r="D12" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E12" s="42">
@@ -5949,36 +5942,35 @@
         <f>F12/E12</f>
         <v>0.000316170728482488</v>
       </c>
-      <c r="H12" s="59">
-        <f>D12/2</f>
+      <c r="H12" s="49">
+        <f>(2*D12*G12)/(2+D12*G12)</f>
+        <v>0.00157960508019014</v>
+      </c>
+      <c r="I12" s="49">
+        <f>1-H12</f>
+        <v>0.99842039491981</v>
+      </c>
+      <c r="J12" s="42">
+        <f>J11*I11</f>
+        <v>98699.2311148191</v>
+      </c>
+      <c r="K12" s="42">
+        <f>J12*H12</f>
+        <v>155.905806879829</v>
+      </c>
+      <c r="L12" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I12" s="49">
-        <f>D12*G12/(1+(D12-H12)*G12)</f>
-        <v>0.00157960508019014</v>
-      </c>
-      <c r="J12" s="49">
-        <f>1-I12</f>
-        <v>0.99842039491981</v>
-      </c>
-      <c r="K12" s="42">
-        <f>K11-L11</f>
-        <v>98703.4922437703</v>
-      </c>
-      <c r="L12" s="42">
-        <f>K12*I12</f>
-        <v>155.912537780768</v>
-      </c>
       <c r="M12" s="42">
-        <f>D12*K13+H12*L12</f>
-        <v>493127.6798744</v>
+        <f>J13*D12+K12*L12</f>
+        <v>493106.391056896</v>
       </c>
       <c r="N12" s="42">
         <f>SUM(M12:$M$25)</f>
-        <v>6675821.41199009</v>
-      </c>
-      <c r="O12" s="60">
-        <f>N12/K12</f>
+        <v>6675533.21007094</v>
+      </c>
+      <c r="O12" s="61">
+        <f>N12/J12</f>
         <v>67.6351085481622</v>
       </c>
       <c r="P12" s="29" t="n"/>
@@ -6007,36 +5999,35 @@
         <f>F13/E13</f>
         <v>0.00122353794267245</v>
       </c>
-      <c r="H13" s="50">
-        <f>D13/2</f>
+      <c r="H13" s="55">
+        <f>(2*D13*G13)/(2+D13*G13)</f>
+        <v>0.006099033715451</v>
+      </c>
+      <c r="I13" s="55">
+        <f>1-H13</f>
+        <v>0.993900966284549</v>
+      </c>
+      <c r="J13" s="39">
+        <f>J12*I12</f>
+        <v>98543.3253079393</v>
+      </c>
+      <c r="K13" s="39">
+        <f>J13*H13</f>
+        <v>601.019063485778</v>
+      </c>
+      <c r="L13" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I13" s="55">
-        <f>D13*G13/(1+(D13-H13)*G13)</f>
-        <v>0.006099033715451</v>
-      </c>
-      <c r="J13" s="55">
-        <f>1-I13</f>
-        <v>0.993900966284549</v>
-      </c>
-      <c r="K13" s="39">
-        <f>K12-L12</f>
-        <v>98547.5797059895</v>
-      </c>
-      <c r="L13" s="39">
-        <f>K13*I13</f>
-        <v>601.045011202925</v>
-      </c>
       <c r="M13" s="39">
-        <f>D13*K14+H13*L13</f>
-        <v>491235.28600194</v>
+        <f>J14*D13+K13*L13</f>
+        <v>491214.078880982</v>
       </c>
       <c r="N13" s="39">
         <f>SUM(M13:$M$25)</f>
-        <v>6182693.73211569</v>
-      </c>
-      <c r="O13" s="56">
-        <f>N13/K13</f>
+        <v>6182426.81901405</v>
+      </c>
+      <c r="O13" s="57">
+        <f>N13/J13</f>
         <v>62.7381590756604</v>
       </c>
       <c r="P13" s="29" t="n"/>
@@ -6047,10 +6038,10 @@
         <f>'Cohorte ficticio'!B53</f>
         <v>20-24</v>
       </c>
-      <c r="C14" s="57" t="n">
+      <c r="C14" s="58" t="n">
         <v>20</v>
       </c>
-      <c r="D14" s="58" t="n">
+      <c r="D14" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E14" s="42">
@@ -6065,36 +6056,35 @@
         <f>F14/E14</f>
         <v>0.00205300339901847</v>
       </c>
-      <c r="H14" s="59">
-        <f>D14/2</f>
+      <c r="H14" s="49">
+        <f>(2*D14*G14)/(2+D14*G14)</f>
+        <v>0.0102126007350377</v>
+      </c>
+      <c r="I14" s="49">
+        <f>1-H14</f>
+        <v>0.989787399264962</v>
+      </c>
+      <c r="J14" s="42">
+        <f>J13*I13</f>
+        <v>97942.3062444535</v>
+      </c>
+      <c r="K14" s="42">
+        <f>J14*H14</f>
+        <v>1000.2456687434</v>
+      </c>
+      <c r="L14" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I14" s="49">
-        <f>D14*G14/(1+(D14-H14)*G14)</f>
-        <v>0.0102126007350377</v>
-      </c>
-      <c r="J14" s="49">
-        <f>1-I14</f>
-        <v>0.989787399264962</v>
-      </c>
-      <c r="K14" s="42">
-        <f>K13-L13</f>
-        <v>97946.5346947866</v>
-      </c>
-      <c r="L14" s="42">
-        <f>K14*I14</f>
-        <v>1000.28885221838</v>
-      </c>
       <c r="M14" s="42">
-        <f>D14*K15+H14*L14</f>
-        <v>487231.951343387</v>
+        <f>J15*D14+K14*L14</f>
+        <v>487210.917050409</v>
       </c>
       <c r="N14" s="42">
         <f>SUM(M14:$M$25)</f>
-        <v>5691458.44611375</v>
-      </c>
-      <c r="O14" s="60">
-        <f>N14/K14</f>
+        <v>5691212.74013307</v>
+      </c>
+      <c r="O14" s="61">
+        <f>N14/J14</f>
         <v>58.1078081409315</v>
       </c>
       <c r="P14" s="29" t="n"/>
@@ -6123,36 +6113,35 @@
         <f>F15/E15</f>
         <v>0.00252753858645077</v>
       </c>
-      <c r="H15" s="50">
-        <f>D15/2</f>
+      <c r="H15" s="55">
+        <f>(2*D15*G15)/(2+D15*G15)</f>
+        <v>0.012558338718025</v>
+      </c>
+      <c r="I15" s="55">
+        <f>1-H15</f>
+        <v>0.987441661281975</v>
+      </c>
+      <c r="J15" s="39">
+        <f>J14*I14</f>
+        <v>96942.0605757101</v>
+      </c>
+      <c r="K15" s="39">
+        <f>J15*H15</f>
+        <v>1217.43123273307</v>
+      </c>
+      <c r="L15" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I15" s="55">
-        <f>D15*G15/(1+(D15-H15)*G15)</f>
-        <v>0.012558338718025</v>
-      </c>
-      <c r="J15" s="55">
-        <f>1-I15</f>
-        <v>0.987441661281975</v>
-      </c>
-      <c r="K15" s="39">
-        <f>K14-L14</f>
-        <v>96946.2458425682</v>
-      </c>
-      <c r="L15" s="39">
-        <f>K15*I15</f>
-        <v>1217.4837927319</v>
-      </c>
       <c r="M15" s="39">
-        <f>D15*K16+H15*L15</f>
-        <v>481687.519731011</v>
+        <f>J16*D15+K15*L15</f>
+        <v>481666.724796718</v>
       </c>
       <c r="N15" s="39">
         <f>SUM(M15:$M$25)</f>
-        <v>5204226.49477037</v>
-      </c>
-      <c r="O15" s="56">
-        <f>N15/K15</f>
+        <v>5204001.82308266</v>
+      </c>
+      <c r="O15" s="57">
+        <f>N15/J15</f>
         <v>53.68156806424</v>
       </c>
       <c r="P15" s="29" t="n"/>
@@ -6163,10 +6152,10 @@
         <f>'Cohorte ficticio'!B55</f>
         <v>30-34</v>
       </c>
-      <c r="C16" s="57" t="n">
+      <c r="C16" s="58" t="n">
         <v>30</v>
       </c>
-      <c r="D16" s="58" t="n">
+      <c r="D16" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E16" s="42">
@@ -6181,36 +6170,35 @@
         <f>F16/E16</f>
         <v>0.00293405593163117</v>
       </c>
-      <c r="H16" s="59">
-        <f>D16/2</f>
+      <c r="H16" s="49">
+        <f>(2*D16*G16)/(2+D16*G16)</f>
+        <v>0.0145634546816713</v>
+      </c>
+      <c r="I16" s="49">
+        <f>1-H16</f>
+        <v>0.985436545318329</v>
+      </c>
+      <c r="J16" s="42">
+        <f>J15*I15</f>
+        <v>95724.6293429771</v>
+      </c>
+      <c r="K16" s="42">
+        <f>J16*H16</f>
+        <v>1394.08130135623</v>
+      </c>
+      <c r="L16" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I16" s="49">
-        <f>D16*G16/(1+(D16-H16)*G16)</f>
-        <v>0.0145634546816713</v>
-      </c>
-      <c r="J16" s="49">
-        <f>1-I16</f>
-        <v>0.985436545318329</v>
-      </c>
-      <c r="K16" s="42">
-        <f>K15-L15</f>
-        <v>95728.7620498363</v>
-      </c>
-      <c r="L16" s="42">
-        <f>K16*I16</f>
-        <v>1394.14148784529</v>
-      </c>
       <c r="M16" s="42">
-        <f>D16*K17+H16*L16</f>
-        <v>475158.456529569</v>
+        <f>J17*D16+K16*L16</f>
+        <v>475137.943461495</v>
       </c>
       <c r="N16" s="42">
         <f>SUM(M16:$M$25)</f>
-        <v>4722538.97503936</v>
-      </c>
-      <c r="O16" s="60">
-        <f>N16/K16</f>
+        <v>4722335.09828594</v>
+      </c>
+      <c r="O16" s="61">
+        <f>N16/J16</f>
         <v>49.3324981323879</v>
       </c>
       <c r="P16" s="29" t="n"/>
@@ -6239,36 +6227,35 @@
         <f>F17/E17</f>
         <v>0.00332166419272473</v>
       </c>
-      <c r="H17" s="50">
-        <f>D17/2</f>
+      <c r="H17" s="55">
+        <f>(2*D17*G17)/(2+D17*G17)</f>
+        <v>0.0164715386631822</v>
+      </c>
+      <c r="I17" s="55">
+        <f>1-H17</f>
+        <v>0.983528461336818</v>
+      </c>
+      <c r="J17" s="39">
+        <f>J16*I16</f>
+        <v>94330.5480416208</v>
+      </c>
+      <c r="K17" s="39">
+        <f>J17*H17</f>
+        <v>1553.76926918673</v>
+      </c>
+      <c r="L17" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I17" s="55">
-        <f>D17*G17/(1+(D17-H17)*G17)</f>
-        <v>0.0164715386631822</v>
-      </c>
-      <c r="J17" s="55">
-        <f>1-I17</f>
-        <v>0.983528461336818</v>
-      </c>
-      <c r="K17" s="39">
-        <f>K16-L16</f>
-        <v>94334.6205619911</v>
-      </c>
-      <c r="L17" s="39">
-        <f>K17*I17</f>
-        <v>1553.83634986346</v>
-      </c>
       <c r="M17" s="39">
-        <f>D17*K18+H17*L17</f>
-        <v>467788.511935297</v>
+        <f>J18*D17+K17*L17</f>
+        <v>467768.317035137</v>
       </c>
       <c r="N17" s="39">
         <f>SUM(M17:$M$25)</f>
-        <v>4247380.51850979</v>
-      </c>
-      <c r="O17" s="56">
-        <f>N17/K17</f>
+        <v>4247197.15482445</v>
+      </c>
+      <c r="O17" s="57">
+        <f>N17/J17</f>
         <v>45.0246207935788</v>
       </c>
       <c r="P17" s="29" t="n"/>
@@ -6279,10 +6266,10 @@
         <f>'Cohorte ficticio'!B57</f>
         <v>40-44</v>
       </c>
-      <c r="C18" s="57" t="n">
+      <c r="C18" s="58" t="n">
         <v>40</v>
       </c>
-      <c r="D18" s="58" t="n">
+      <c r="D18" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E18" s="42">
@@ -6297,37 +6284,36 @@
         <f>F18/E18</f>
         <v>0.00397480590187037</v>
       </c>
-      <c r="H18" s="59">
-        <f>D18/2</f>
+      <c r="H18" s="49">
+        <f>(2*D18*G18)/(2+D18*G18)</f>
+        <v>0.0196784841222791</v>
+      </c>
+      <c r="I18" s="49">
+        <f>1-H18</f>
+        <v>0.980321515877721</v>
+      </c>
+      <c r="J18" s="42">
+        <f>J17*I17</f>
+        <v>92776.7787724341</v>
+      </c>
+      <c r="K18" s="42">
+        <f>J18*H18</f>
+        <v>1825.70636798955</v>
+      </c>
+      <c r="L18" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I18" s="49">
-        <f>D18*G18/(1+(D18-H18)*G18)</f>
-        <v>0.0196784841222791</v>
-      </c>
-      <c r="J18" s="49">
-        <f>1-I18</f>
-        <v>0.980321515877721</v>
-      </c>
-      <c r="K18" s="42">
-        <f>K17-L17</f>
-        <v>92780.7842121276</v>
-      </c>
-      <c r="L18" s="42">
-        <f>K18*I18</f>
-        <v>1825.78518897096</v>
-      </c>
       <c r="M18" s="42">
-        <f>D18*K19+H18*L18</f>
-        <v>459339.458088211</v>
+        <f>J19*D18+K18*L18</f>
+        <v>459319.627942197</v>
       </c>
       <c r="N18" s="42">
         <f>SUM(M18:$M$25)</f>
-        <v>3779592.00657449</v>
-      </c>
-      <c r="O18" s="60">
-        <f>N18/K18</f>
-        <v>40.7367973731833</v>
+        <v>3779428.83778931</v>
+      </c>
+      <c r="O18" s="61">
+        <f>N18/J18</f>
+        <v>40.7367973731834</v>
       </c>
       <c r="P18" s="29" t="n"/>
     </row>
@@ -6355,36 +6341,35 @@
         <f>F19/E19</f>
         <v>0.00535757605711496</v>
       </c>
-      <c r="H19" s="50">
-        <f>D19/2</f>
+      <c r="H19" s="55">
+        <f>(2*D19*G19)/(2+D19*G19)</f>
+        <v>0.0264338271864941</v>
+      </c>
+      <c r="I19" s="55">
+        <f>1-H19</f>
+        <v>0.973566172813506</v>
+      </c>
+      <c r="J19" s="39">
+        <f>J18*I18</f>
+        <v>90951.0724044446</v>
+      </c>
+      <c r="K19" s="39">
+        <f>J19*H19</f>
+        <v>2404.1849303654</v>
+      </c>
+      <c r="L19" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I19" s="55">
-        <f>D19*G19/(1+(D19-H19)*G19)</f>
-        <v>0.0264338271864941</v>
-      </c>
-      <c r="J19" s="55">
-        <f>1-I19</f>
-        <v>0.973566172813506</v>
-      </c>
-      <c r="K19" s="39">
-        <f>K18-L18</f>
-        <v>90954.9990231566</v>
-      </c>
-      <c r="L19" s="39">
-        <f>K19*I19</f>
-        <v>2404.28872592586</v>
-      </c>
       <c r="M19" s="39">
-        <f>D19*K20+H19*L19</f>
-        <v>448764.273300968</v>
+        <f>J20*D19+K19*L19</f>
+        <v>448744.899696309</v>
       </c>
       <c r="N19" s="39">
         <f>SUM(M19:$M$25)</f>
-        <v>3320252.54848628</v>
-      </c>
-      <c r="O19" s="56">
-        <f>N19/K19</f>
+        <v>3320109.20984711</v>
+      </c>
+      <c r="O19" s="57">
+        <f>N19/J19</f>
         <v>36.5043437320137</v>
       </c>
       <c r="P19" s="29" t="n"/>
@@ -6395,10 +6380,10 @@
         <f>'Cohorte ficticio'!B59</f>
         <v>50-54</v>
       </c>
-      <c r="C20" s="57" t="n">
+      <c r="C20" s="58" t="n">
         <v>50</v>
       </c>
-      <c r="D20" s="58" t="n">
+      <c r="D20" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E20" s="42">
@@ -6413,36 +6398,35 @@
         <f>F20/E20</f>
         <v>0.00695707719003293</v>
       </c>
-      <c r="H20" s="59">
-        <f>D20/2</f>
+      <c r="H20" s="49">
+        <f>(2*D20*G20)/(2+D20*G20)</f>
+        <v>0.0341907173015411</v>
+      </c>
+      <c r="I20" s="49">
+        <f>1-H20</f>
+        <v>0.965809282698459</v>
+      </c>
+      <c r="J20" s="42">
+        <f>J19*I19</f>
+        <v>88546.8874740792</v>
+      </c>
+      <c r="K20" s="42">
+        <f>J20*H20</f>
+        <v>3027.48159755761</v>
+      </c>
+      <c r="L20" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I20" s="49">
-        <f>D20*G20/(1+(D20-H20)*G20)</f>
-        <v>0.0341907173015411</v>
-      </c>
-      <c r="J20" s="49">
-        <f>1-I20</f>
-        <v>0.965809282698459</v>
-      </c>
-      <c r="K20" s="42">
-        <f>K19-L19</f>
-        <v>88550.7102972308</v>
-      </c>
-      <c r="L20" s="42">
-        <f>K20*I20</f>
-        <v>3027.61230262328</v>
-      </c>
       <c r="M20" s="42">
-        <f>D20*K21+H20*L20</f>
-        <v>435184.520729596</v>
+        <f>J21*D20+K20*L20</f>
+        <v>435165.733376502</v>
       </c>
       <c r="N20" s="42">
         <f>SUM(M20:$M$25)</f>
-        <v>2871488.27518531</v>
-      </c>
-      <c r="O20" s="60">
-        <f>N20/K20</f>
+        <v>2871364.3101508</v>
+      </c>
+      <c r="O20" s="61">
+        <f>N20/J20</f>
         <v>32.4276142511655</v>
       </c>
       <c r="P20" s="29" t="n"/>
@@ -6471,36 +6455,35 @@
         <f>F21/E21</f>
         <v>0.00991633642442753</v>
       </c>
-      <c r="H21" s="50">
-        <f>D21/2</f>
+      <c r="H21" s="55">
+        <f>(2*D21*G21)/(2+D21*G21)</f>
+        <v>0.0483822455622269</v>
+      </c>
+      <c r="I21" s="55">
+        <f>1-H21</f>
+        <v>0.951617754437773</v>
+      </c>
+      <c r="J21" s="39">
+        <f>J20*I20</f>
+        <v>85519.4058765216</v>
+      </c>
+      <c r="K21" s="39">
+        <f>J21*H21</f>
+        <v>4137.62089545362</v>
+      </c>
+      <c r="L21" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I21" s="55">
-        <f>D21*G21/(1+(D21-H21)*G21)</f>
-        <v>0.0483822455622269</v>
-      </c>
-      <c r="J21" s="55">
-        <f>1-I21</f>
-        <v>0.951617754437773</v>
-      </c>
-      <c r="K21" s="39">
-        <f>K20-L20</f>
-        <v>85523.0979946075</v>
-      </c>
-      <c r="L21" s="39">
-        <f>K21*I21</f>
-        <v>4137.79952841749</v>
-      </c>
       <c r="M21" s="39">
-        <f>D21*K22+H21*L21</f>
-        <v>417270.991151994</v>
+        <f>J22*D21+K21*L21</f>
+        <v>417252.977143974</v>
       </c>
       <c r="N21" s="39">
         <f>SUM(M21:$M$25)</f>
-        <v>2436303.75445572</v>
-      </c>
-      <c r="O21" s="56">
-        <f>N21/K21</f>
+        <v>2436198.5767743</v>
+      </c>
+      <c r="O21" s="57">
+        <f>N21/J21</f>
         <v>28.487084911369</v>
       </c>
       <c r="P21" s="29" t="n"/>
@@ -6511,10 +6494,10 @@
         <f>'Cohorte ficticio'!B61</f>
         <v>60-64</v>
       </c>
-      <c r="C22" s="57" t="n">
+      <c r="C22" s="58" t="n">
         <v>60</v>
       </c>
-      <c r="D22" s="58" t="n">
+      <c r="D22" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E22" s="42">
@@ -6529,36 +6512,35 @@
         <f>F22/E22</f>
         <v>0.0135201532364292</v>
       </c>
-      <c r="H22" s="59">
-        <f>D22/2</f>
+      <c r="H22" s="49">
+        <f>(2*D22*G22)/(2+D22*G22)</f>
+        <v>0.0653905408508544</v>
+      </c>
+      <c r="I22" s="49">
+        <f>1-H22</f>
+        <v>0.934609459149146</v>
+      </c>
+      <c r="J22" s="42">
+        <f>J21*I21</f>
+        <v>81381.784981068</v>
+      </c>
+      <c r="K22" s="42">
+        <f>J22*H22</f>
+        <v>5321.59893531998</v>
+      </c>
+      <c r="L22" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I22" s="49">
-        <f>D22*G22/(1+(D22-H22)*G22)</f>
-        <v>0.0653905408508544</v>
-      </c>
-      <c r="J22" s="49">
-        <f>1-I22</f>
-        <v>0.934609459149146</v>
-      </c>
-      <c r="K22" s="42">
-        <f>K21-L21</f>
-        <v>81385.29846619</v>
-      </c>
-      <c r="L22" s="42">
-        <f>K22*I22</f>
-        <v>5321.82868401238</v>
-      </c>
       <c r="M22" s="42">
-        <f>D22*K23+H22*L22</f>
-        <v>393621.920620919</v>
+        <f>J23*D22+K22*L22</f>
+        <v>393604.92756704</v>
       </c>
       <c r="N22" s="42">
         <f>SUM(M22:$M$25)</f>
-        <v>2019032.76330372</v>
-      </c>
-      <c r="O22" s="60">
-        <f>N22/K22</f>
+        <v>2018945.59963033</v>
+      </c>
+      <c r="O22" s="61">
+        <f>N22/J22</f>
         <v>24.8083228955963</v>
       </c>
       <c r="P22" s="29" t="n"/>
@@ -6587,36 +6569,35 @@
         <f>F23/E23</f>
         <v>0.0183639764635371</v>
       </c>
-      <c r="H23" s="50">
-        <f>D23/2</f>
+      <c r="H23" s="55">
+        <f>(2*D23*G23)/(2+D23*G23)</f>
+        <v>0.0877894727876391</v>
+      </c>
+      <c r="I23" s="55">
+        <f>1-H23</f>
+        <v>0.912210527212361</v>
+      </c>
+      <c r="J23" s="39">
+        <f>J22*I22</f>
+        <v>76060.186045748</v>
+      </c>
+      <c r="K23" s="39">
+        <f>J23*H23</f>
+        <v>6677.28363308596</v>
+      </c>
+      <c r="L23" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I23" s="55">
-        <f>D23*G23/(1+(D23-H23)*G23)</f>
-        <v>0.0877894727876391</v>
-      </c>
-      <c r="J23" s="55">
-        <f>1-I23</f>
-        <v>0.912210527212361</v>
-      </c>
-      <c r="K23" s="39">
-        <f>K22-L22</f>
-        <v>76063.4697821776</v>
-      </c>
-      <c r="L23" s="39">
-        <f>K23*I23</f>
-        <v>6677.57191057589</v>
-      </c>
       <c r="M23" s="39">
-        <f>D23*K24+H23*L23</f>
-        <v>363623.419134448</v>
+        <f>J24*D23+K23*L23</f>
+        <v>363607.721146025</v>
       </c>
       <c r="N23" s="39">
         <f>SUM(M23:$M$25)</f>
-        <v>1625410.8426828</v>
-      </c>
-      <c r="O23" s="56">
-        <f>N23/K23</f>
+        <v>1625340.67206329</v>
+      </c>
+      <c r="O23" s="57">
+        <f>N23/J23</f>
         <v>21.3691387907688</v>
       </c>
       <c r="P23" s="29" t="n"/>
@@ -6627,10 +6608,10 @@
         <f>'Cohorte ficticio'!B63</f>
         <v>70-74</v>
       </c>
-      <c r="C24" s="57" t="n">
+      <c r="C24" s="58" t="n">
         <v>70</v>
       </c>
-      <c r="D24" s="58" t="n">
+      <c r="D24" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E24" s="42">
@@ -6645,36 +6626,35 @@
         <f>F24/E24</f>
         <v>0.0270520906873422</v>
       </c>
-      <c r="H24" s="59">
-        <f>D24/2</f>
+      <c r="H24" s="49">
+        <f>(2*D24*G24)/(2+D24*G24)</f>
+        <v>0.126692229249138</v>
+      </c>
+      <c r="I24" s="49">
+        <f>1-H24</f>
+        <v>0.873307770750862</v>
+      </c>
+      <c r="J24" s="42">
+        <f>J23*I23</f>
+        <v>69382.902412662</v>
+      </c>
+      <c r="K24" s="42">
+        <f>J24*H24</f>
+        <v>8790.27457843555</v>
+      </c>
+      <c r="L24" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I24" s="49">
-        <f>D24*G24/(1+(D24-H24)*G24)</f>
-        <v>0.126692229249138</v>
-      </c>
-      <c r="J24" s="49">
-        <f>1-I24</f>
-        <v>0.873307770750862</v>
-      </c>
-      <c r="K24" s="42">
-        <f>K23-L23</f>
-        <v>69385.8978716017</v>
-      </c>
-      <c r="L24" s="42">
-        <f>K24*I24</f>
-        <v>8790.65407980624</v>
-      </c>
       <c r="M24" s="42">
-        <f>D24*K25+H24*L24</f>
-        <v>324952.854158493</v>
+        <f>J25*D24+K24*L24</f>
+        <v>324938.825617221</v>
       </c>
       <c r="N24" s="42">
         <f>SUM(M24:$M$25)</f>
-        <v>1261787.42354835</v>
-      </c>
-      <c r="O24" s="60">
-        <f>N24/K24</f>
+        <v>1261732.95091726</v>
+      </c>
+      <c r="O24" s="61">
+        <f>N24/J24</f>
         <v>18.1850701980291</v>
       </c>
       <c r="P24" s="29" t="n"/>
@@ -6705,36 +6685,35 @@
         <f>F25/E25</f>
         <v>0.0646808366937823</v>
       </c>
-      <c r="H25" s="61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I25" s="55" t="n">
+      <c r="H25" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="J25" s="55">
-        <f>1-I25</f>
+      <c r="I25" s="55">
+        <f>1-H25</f>
         <v>0</v>
       </c>
+      <c r="J25" s="39">
+        <f>J24*I24</f>
+        <v>60592.6278342265</v>
+      </c>
       <c r="K25" s="39">
-        <f>K24-L24</f>
-        <v>60595.2437917955</v>
-      </c>
-      <c r="L25" s="39">
-        <f>K25*I25</f>
-        <v>60595.2437917955</v>
+        <f>J25*H25</f>
+        <v>60592.6278342265</v>
+      </c>
+      <c r="L25" s="56">
+        <f>1/G25</f>
+        <v>15.4605297506321</v>
       </c>
       <c r="M25" s="39">
-        <f>K25/G25</f>
-        <v>936834.569389862</v>
+        <f>K25*L25</f>
+        <v>936794.12530004</v>
       </c>
       <c r="N25" s="39">
         <f>SUM(M25:$M$25)</f>
-        <v>936834.569389862</v>
-      </c>
-      <c r="O25" s="56">
-        <f>N25/K25</f>
+        <v>936794.12530004</v>
+      </c>
+      <c r="O25" s="57">
+        <f>N25/J25</f>
         <v>15.4605297506321</v>
       </c>
       <c r="P25" s="29" t="n"/>
@@ -6765,7 +6744,7 @@
         </is>
       </c>
       <c r="E27" s="48">
-        <f>ROUND(SUM(L9:L25)-D5,6)</f>
+        <f>ROUND(SUM(K9:K25)-D5,6)</f>
         <v>0</v>
       </c>
       <c r="F27" s="35" t="inlineStr">
@@ -6786,12 +6765,12 @@
       <c r="A28" s="29" t="n"/>
       <c r="B28" s="62" t="inlineStr">
         <is>
-          <t>q0 (mortalidad infantil, por mil)</t>
-        </is>
-      </c>
-      <c r="E28" s="56">
-        <f>I9*1000</f>
-        <v>9.92937335308912</v>
+          <t>q0 (por mil)</t>
+        </is>
+      </c>
+      <c r="E28" s="57">
+        <f>H9*1000</f>
+        <v>9.97176113009477</v>
       </c>
       <c r="F28" s="29" t="n"/>
       <c r="G28" s="29" t="n"/>
@@ -6905,11 +6884,11 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="9" customWidth="1" min="15" max="15"/>
@@ -7025,7 +7004,7 @@
       <c r="A6" s="29" t="n"/>
       <c r="B6" s="35" t="inlineStr">
         <is>
-          <t>nMx = D/P;  nqx = n·nMx / (1 + (n − nax)·nMx);  lx+n = lx·(1 − nqx);  ndx = lx − lx+n;  nLx = n·lx+n + nax·ndx;  Tx = suma de nLx hacia abajo;  ex = Tx/lx.  Grupo abierto 75+: q = 1 y L = l/M.</t>
+          <t>nmx = D/P;  nqx = (2·n·nmx) / (2 + n·nmx);  npx = 1 − nqx;  lx+n = lx·npx;  ndx = lx·nqx;  nLx = lx+n·n + ndx·nAx;  Tx = suma de nLx hacia abajo;  ex = Tx/lx.</t>
         </is>
       </c>
       <c r="P6" s="29" t="n"/>
@@ -7034,7 +7013,7 @@
       <c r="A7" s="29" t="n"/>
       <c r="B7" s="35" t="inlineStr">
         <is>
-          <t>nax: para 0 y 1-4, Coale-Demeny según la mortalidad infantil y el sexo (en ambos sexos, el promedio de hombres y mujeres); n/2 en los demás grupos. Valores sin redondear.</t>
+          <t>nAx: 0.12 en la edad 0, 1.5 en 1-4 y 2.5 en los demás grupos (los valores del Cuadro 4.3 del ejemplo de la profesora). En el grupo abierto 75+: nqx = 1 y nAx = 1/nmx.</t>
         </is>
       </c>
       <c r="P7" s="29" t="n"/>
@@ -7068,32 +7047,32 @@
       </c>
       <c r="G8" s="37" t="inlineStr">
         <is>
-          <t>nMx</t>
+          <t>nmx</t>
         </is>
       </c>
       <c r="H8" s="37" t="inlineStr">
         <is>
-          <t>nax</t>
+          <t>nqx</t>
         </is>
       </c>
       <c r="I8" s="37" t="inlineStr">
         <is>
-          <t>nqx</t>
+          <t>npx</t>
         </is>
       </c>
       <c r="J8" s="37" t="inlineStr">
         <is>
-          <t>npx</t>
+          <t>lx</t>
         </is>
       </c>
       <c r="K8" s="37" t="inlineStr">
         <is>
-          <t>lx</t>
+          <t>ndx</t>
         </is>
       </c>
       <c r="L8" s="37" t="inlineStr">
         <is>
-          <t>ndx</t>
+          <t>nAx</t>
         </is>
       </c>
       <c r="M8" s="37" t="inlineStr">
@@ -7137,37 +7116,36 @@
         <f>F9/E9</f>
         <v>0.00787653360180393</v>
       </c>
-      <c r="H9" s="50">
-        <f>IF($G$9&gt;=0.107,0.35,0.053+2.8*$G$9)</f>
-        <v>0.075054294085051</v>
+      <c r="H9" s="55">
+        <f>(2*D9*G9)/(2+D9*G9)</f>
+        <v>0.00784563539639034</v>
       </c>
       <c r="I9" s="55">
-        <f>D9*G9/(1+(D9-H9)*G9)</f>
-        <v>0.00781956520783196</v>
-      </c>
-      <c r="J9" s="55">
-        <f>1-I9</f>
-        <v>0.992180434792168</v>
-      </c>
-      <c r="K9" s="39">
+        <f>1-H9</f>
+        <v>0.99215436460361</v>
+      </c>
+      <c r="J9" s="39">
         <f>$D$5</f>
         <v>100000</v>
       </c>
-      <c r="L9" s="39">
-        <f>K9*I9</f>
-        <v>781.956520783196</v>
+      <c r="K9" s="39">
+        <f>J9*H9</f>
+        <v>784.563539639034</v>
+      </c>
+      <c r="L9" s="56" t="n">
+        <v>0.12</v>
       </c>
       <c r="M9" s="39">
-        <f>D9*K10+H9*L9</f>
-        <v>99276.7326738894</v>
+        <f>J10*D9+K9*L9</f>
+        <v>99309.5840851177</v>
       </c>
       <c r="N9" s="39">
         <f>SUM(M9:$M$25)</f>
-        <v>8392453.67809822</v>
-      </c>
-      <c r="O9" s="56">
-        <f>N9/K9</f>
-        <v>83.9245367809822</v>
+        <v>8392264.01604984</v>
+      </c>
+      <c r="O9" s="57">
+        <f>N9/J9</f>
+        <v>83.9226401604984</v>
       </c>
       <c r="P9" s="29" t="n"/>
     </row>
@@ -7177,10 +7155,10 @@
         <f>'Cohorte ficticio'!B49</f>
         <v>1-4</v>
       </c>
-      <c r="C10" s="57" t="n">
+      <c r="C10" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="58" t="n">
+      <c r="D10" s="59" t="n">
         <v>4</v>
       </c>
       <c r="E10" s="42">
@@ -7195,37 +7173,36 @@
         <f>F10/E10</f>
         <v>0.000426722126857265</v>
       </c>
-      <c r="H10" s="59">
-        <f>IF($G$9&gt;=0.107,1.361,1.522-1.518*$G$9)</f>
-        <v>1.51004342199246</v>
+      <c r="H10" s="49">
+        <f>(2*D10*G10)/(2+D10*G10)</f>
+        <v>0.00170543301542195</v>
       </c>
       <c r="I10" s="49">
-        <f>D10*G10/(1+(D10-H10)*G10)</f>
-        <v>0.00170507682993444</v>
-      </c>
-      <c r="J10" s="49">
-        <f>1-I10</f>
-        <v>0.998294923170066</v>
+        <f>1-H10</f>
+        <v>0.998294566984578</v>
+      </c>
+      <c r="J10" s="42">
+        <f>J9*I9</f>
+        <v>99215.436460361</v>
       </c>
       <c r="K10" s="42">
-        <f>K9-L9</f>
-        <v>99218.0434792168</v>
-      </c>
-      <c r="L10" s="42">
-        <f>K10*I10</f>
-        <v>169.174387047841</v>
+        <f>J10*H10</f>
+        <v>169.205280978999</v>
+      </c>
+      <c r="L10" s="60" t="n">
+        <v>1.5</v>
       </c>
       <c r="M10" s="42">
-        <f>D10*K11+H10*L10</f>
-        <v>396450.937039007</v>
+        <f>J11*D10+K10*L10</f>
+        <v>396438.732638996</v>
       </c>
       <c r="N10" s="42">
         <f>SUM(M10:$M$25)</f>
-        <v>8293176.94542433</v>
-      </c>
-      <c r="O10" s="60">
-        <f>N10/K10</f>
-        <v>83.5853707109383</v>
+        <v>8292954.43196473</v>
+      </c>
+      <c r="O10" s="61">
+        <f>N10/J10</f>
+        <v>83.585324298583</v>
       </c>
       <c r="P10" s="29" t="n"/>
     </row>
@@ -7253,36 +7230,35 @@
         <f>F11/E11</f>
         <v>0.000173842647861825</v>
       </c>
-      <c r="H11" s="50">
-        <f>D11/2</f>
+      <c r="H11" s="55">
+        <f>(2*D11*G11)/(2+D11*G11)</f>
+        <v>0.000868835637589636</v>
+      </c>
+      <c r="I11" s="55">
+        <f>1-H11</f>
+        <v>0.99913116436241</v>
+      </c>
+      <c r="J11" s="39">
+        <f>J10*I10</f>
+        <v>99046.231179382</v>
+      </c>
+      <c r="K11" s="39">
+        <f>J11*H11</f>
+        <v>86.0548954175888</v>
+      </c>
+      <c r="L11" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I11" s="55">
-        <f>D11*G11/(1+(D11-H11)*G11)</f>
-        <v>0.000868835637589636</v>
-      </c>
-      <c r="J11" s="55">
-        <f>1-I11</f>
-        <v>0.99913116436241</v>
-      </c>
-      <c r="K11" s="39">
-        <f>K10-L10</f>
-        <v>99048.869092169</v>
-      </c>
-      <c r="L11" s="39">
-        <f>K11*I11</f>
-        <v>86.057187330227</v>
-      </c>
       <c r="M11" s="39">
-        <f>D11*K12+H11*L11</f>
-        <v>495029.202492519</v>
+        <f>J12*D11+K11*L11</f>
+        <v>495016.018658366</v>
       </c>
       <c r="N11" s="39">
         <f>SUM(M11:$M$25)</f>
-        <v>7896726.00838533</v>
-      </c>
-      <c r="O11" s="56">
-        <f>N11/K11</f>
+        <v>7896515.69932573</v>
+      </c>
+      <c r="O11" s="57">
+        <f>N11/J11</f>
         <v>79.7255544738942</v>
       </c>
       <c r="P11" s="29" t="n"/>
@@ -7293,10 +7269,10 @@
         <f>'Cohorte ficticio'!B51</f>
         <v>10-14</v>
       </c>
-      <c r="C12" s="57" t="n">
+      <c r="C12" s="58" t="n">
         <v>10</v>
       </c>
-      <c r="D12" s="58" t="n">
+      <c r="D12" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E12" s="42">
@@ -7311,36 +7287,35 @@
         <f>F12/E12</f>
         <v>0.00024533053283636</v>
       </c>
-      <c r="H12" s="59">
-        <f>D12/2</f>
+      <c r="H12" s="49">
+        <f>(2*D12*G12)/(2+D12*G12)</f>
+        <v>0.00122590078694863</v>
+      </c>
+      <c r="I12" s="49">
+        <f>1-H12</f>
+        <v>0.998774099213051</v>
+      </c>
+      <c r="J12" s="42">
+        <f>J11*I11</f>
+        <v>98960.1762839644</v>
+      </c>
+      <c r="K12" s="42">
+        <f>J12*H12</f>
+        <v>121.315357983087</v>
+      </c>
+      <c r="L12" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I12" s="49">
-        <f>D12*G12/(1+(D12-H12)*G12)</f>
-        <v>0.00122590078694863</v>
-      </c>
-      <c r="J12" s="49">
-        <f>1-I12</f>
-        <v>0.998774099213051</v>
-      </c>
-      <c r="K12" s="42">
-        <f>K11-L11</f>
-        <v>98962.8119048388</v>
-      </c>
-      <c r="L12" s="42">
-        <f>K12*I12</f>
-        <v>121.318588992791</v>
-      </c>
       <c r="M12" s="42">
-        <f>D12*K13+H12*L12</f>
-        <v>494510.763051712</v>
+        <f>J13*D12+K12*L12</f>
+        <v>494497.593024864</v>
       </c>
       <c r="N12" s="42">
         <f>SUM(M12:$M$25)</f>
-        <v>7401696.80589281</v>
-      </c>
-      <c r="O12" s="60">
-        <f>N12/K12</f>
+        <v>7401499.68066736</v>
+      </c>
+      <c r="O12" s="61">
+        <f>N12/J12</f>
         <v>74.7927091341157</v>
       </c>
       <c r="P12" s="29" t="n"/>
@@ -7369,36 +7344,35 @@
         <f>F13/E13</f>
         <v>0.000423636121384722</v>
       </c>
-      <c r="H13" s="50">
-        <f>D13/2</f>
+      <c r="H13" s="55">
+        <f>(2*D13*G13)/(2+D13*G13)</f>
+        <v>0.00211593963577265</v>
+      </c>
+      <c r="I13" s="55">
+        <f>1-H13</f>
+        <v>0.997884060364227</v>
+      </c>
+      <c r="J13" s="39">
+        <f>J12*I12</f>
+        <v>98838.8609259813</v>
+      </c>
+      <c r="K13" s="39">
+        <f>J13*H13</f>
+        <v>209.137063387905</v>
+      </c>
+      <c r="L13" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I13" s="55">
-        <f>D13*G13/(1+(D13-H13)*G13)</f>
-        <v>0.00211593963577265</v>
-      </c>
-      <c r="J13" s="55">
-        <f>1-I13</f>
-        <v>0.997884060364227</v>
-      </c>
-      <c r="K13" s="39">
-        <f>K12-L12</f>
-        <v>98841.493315846</v>
-      </c>
-      <c r="L13" s="39">
-        <f>K13*I13</f>
-        <v>209.142633365956</v>
-      </c>
       <c r="M13" s="39">
-        <f>D13*K14+H13*L13</f>
-        <v>493684.609995815</v>
+        <f>J14*D13+K13*L13</f>
+        <v>493671.461971437</v>
       </c>
       <c r="N13" s="39">
         <f>SUM(M13:$M$25)</f>
-        <v>6907186.0428411</v>
-      </c>
-      <c r="O13" s="56">
-        <f>N13/K13</f>
+        <v>6907002.0876425</v>
+      </c>
+      <c r="O13" s="57">
+        <f>N13/J13</f>
         <v>69.881441600334</v>
       </c>
       <c r="P13" s="29" t="n"/>
@@ -7409,10 +7383,10 @@
         <f>'Cohorte ficticio'!B53</f>
         <v>20-24</v>
       </c>
-      <c r="C14" s="57" t="n">
+      <c r="C14" s="58" t="n">
         <v>20</v>
       </c>
-      <c r="D14" s="58" t="n">
+      <c r="D14" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E14" s="42">
@@ -7427,36 +7401,35 @@
         <f>F14/E14</f>
         <v>0.000523928626871653</v>
       </c>
-      <c r="H14" s="59">
-        <f>D14/2</f>
+      <c r="H14" s="49">
+        <f>(2*D14*G14)/(2+D14*G14)</f>
+        <v>0.00261621635774848</v>
+      </c>
+      <c r="I14" s="49">
+        <f>1-H14</f>
+        <v>0.997383783642252</v>
+      </c>
+      <c r="J14" s="42">
+        <f>J13*I13</f>
+        <v>98629.7238625934</v>
+      </c>
+      <c r="K14" s="42">
+        <f>J14*H14</f>
+        <v>258.036696929532</v>
+      </c>
+      <c r="L14" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I14" s="49">
-        <f>D14*G14/(1+(D14-H14)*G14)</f>
-        <v>0.00261621635774848</v>
-      </c>
-      <c r="J14" s="49">
-        <f>1-I14</f>
-        <v>0.997383783642252</v>
-      </c>
-      <c r="K14" s="42">
-        <f>K13-L13</f>
-        <v>98632.35068248</v>
-      </c>
-      <c r="L14" s="42">
-        <f>K14*I14</f>
-        <v>258.043569258689</v>
-      </c>
       <c r="M14" s="42">
-        <f>D14*K15+H14*L14</f>
-        <v>492516.644489253</v>
+        <f>J15*D14+K14*L14</f>
+        <v>492503.527570643</v>
       </c>
       <c r="N14" s="42">
         <f>SUM(M14:$M$25)</f>
-        <v>6413501.43284528</v>
-      </c>
-      <c r="O14" s="60">
-        <f>N14/K14</f>
+        <v>6413330.62567106</v>
+      </c>
+      <c r="O14" s="61">
+        <f>N14/J14</f>
         <v>65.0243189832492</v>
       </c>
       <c r="P14" s="29" t="n"/>
@@ -7485,36 +7458,35 @@
         <f>F15/E15</f>
         <v>0.00068195908012502</v>
       </c>
-      <c r="H15" s="50">
-        <f>D15/2</f>
+      <c r="H15" s="55">
+        <f>(2*D15*G15)/(2+D15*G15)</f>
+        <v>0.00340399194259029</v>
+      </c>
+      <c r="I15" s="55">
+        <f>1-H15</f>
+        <v>0.99659600805741</v>
+      </c>
+      <c r="J15" s="39">
+        <f>J14*I14</f>
+        <v>98371.6871656639</v>
+      </c>
+      <c r="K15" s="39">
+        <f>J15*H15</f>
+        <v>334.856430490933</v>
+      </c>
+      <c r="L15" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I15" s="55">
-        <f>D15*G15/(1+(D15-H15)*G15)</f>
-        <v>0.00340399194259029</v>
-      </c>
-      <c r="J15" s="55">
-        <f>1-I15</f>
-        <v>0.99659600805741</v>
-      </c>
-      <c r="K15" s="39">
-        <f>K14-L14</f>
-        <v>98374.3071132213</v>
-      </c>
-      <c r="L15" s="39">
-        <f>K15*I15</f>
-        <v>334.865348771308</v>
-      </c>
       <c r="M15" s="39">
-        <f>D15*K16+H15*L15</f>
-        <v>491034.372194178</v>
+        <f>J16*D15+K15*L15</f>
+        <v>491021.294752092</v>
       </c>
       <c r="N15" s="39">
         <f>SUM(M15:$M$25)</f>
-        <v>5920984.78835603</v>
-      </c>
-      <c r="O15" s="56">
-        <f>N15/K15</f>
+        <v>5920827.09810042</v>
+      </c>
+      <c r="O15" s="57">
+        <f>N15/J15</f>
         <v>60.1883252050907</v>
       </c>
       <c r="P15" s="29" t="n"/>
@@ -7525,10 +7497,10 @@
         <f>'Cohorte ficticio'!B55</f>
         <v>30-34</v>
       </c>
-      <c r="C16" s="57" t="n">
+      <c r="C16" s="58" t="n">
         <v>30</v>
       </c>
-      <c r="D16" s="58" t="n">
+      <c r="D16" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E16" s="42">
@@ -7543,36 +7515,35 @@
         <f>F16/E16</f>
         <v>0.000881621630898313</v>
       </c>
-      <c r="H16" s="59">
-        <f>D16/2</f>
+      <c r="H16" s="49">
+        <f>(2*D16*G16)/(2+D16*G16)</f>
+        <v>0.0043984138125945</v>
+      </c>
+      <c r="I16" s="49">
+        <f>1-H16</f>
+        <v>0.995601586187406</v>
+      </c>
+      <c r="J16" s="42">
+        <f>J15*I15</f>
+        <v>98036.8307351729</v>
+      </c>
+      <c r="K16" s="42">
+        <f>J16*H16</f>
+        <v>431.206550448574</v>
+      </c>
+      <c r="L16" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I16" s="49">
-        <f>D16*G16/(1+(D16-H16)*G16)</f>
-        <v>0.0043984138125945</v>
-      </c>
-      <c r="J16" s="49">
-        <f>1-I16</f>
-        <v>0.995601586187406</v>
-      </c>
-      <c r="K16" s="42">
-        <f>K15-L15</f>
-        <v>98039.44176445</v>
-      </c>
-      <c r="L16" s="42">
-        <f>K16*I16</f>
-        <v>431.218034835811</v>
-      </c>
       <c r="M16" s="42">
-        <f>D16*K17+H16*L16</f>
-        <v>489119.163735161</v>
+        <f>J17*D16+K16*L16</f>
+        <v>489106.137299743</v>
       </c>
       <c r="N16" s="42">
         <f>SUM(M16:$M$25)</f>
-        <v>5429950.41616185</v>
-      </c>
-      <c r="O16" s="60">
-        <f>N16/K16</f>
+        <v>5429805.80334833</v>
+      </c>
+      <c r="O16" s="61">
+        <f>N16/J16</f>
         <v>55.3853665263402</v>
       </c>
       <c r="P16" s="29" t="n"/>
@@ -7601,36 +7572,35 @@
         <f>F17/E17</f>
         <v>0.00113646773848299</v>
       </c>
-      <c r="H17" s="50">
-        <f>D17/2</f>
+      <c r="H17" s="55">
+        <f>(2*D17*G17)/(2+D17*G17)</f>
+        <v>0.00566623994517447</v>
+      </c>
+      <c r="I17" s="55">
+        <f>1-H17</f>
+        <v>0.994333760054826</v>
+      </c>
+      <c r="J17" s="39">
+        <f>J16*I16</f>
+        <v>97605.6241847244</v>
+      </c>
+      <c r="K17" s="39">
+        <f>J17*H17</f>
+        <v>553.056886629172</v>
+      </c>
+      <c r="L17" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I17" s="55">
-        <f>D17*G17/(1+(D17-H17)*G17)</f>
-        <v>0.00566623994517447</v>
-      </c>
-      <c r="J17" s="55">
-        <f>1-I17</f>
-        <v>0.994333760054826</v>
-      </c>
-      <c r="K17" s="39">
-        <f>K16-L16</f>
-        <v>97608.2237296142</v>
-      </c>
-      <c r="L17" s="39">
-        <f>K17*I17</f>
-        <v>553.071616274266</v>
-      </c>
       <c r="M17" s="39">
-        <f>D17*K18+H17*L17</f>
-        <v>486658.439607385</v>
+        <f>J18*D17+K17*L17</f>
+        <v>486645.478707049</v>
       </c>
       <c r="N17" s="39">
         <f>SUM(M17:$M$25)</f>
-        <v>4940831.25242669</v>
-      </c>
-      <c r="O17" s="56">
-        <f>N17/K17</f>
+        <v>4940699.66604858</v>
+      </c>
+      <c r="O17" s="57">
+        <f>N17/J17</f>
         <v>50.6190058955826</v>
       </c>
       <c r="P17" s="29" t="n"/>
@@ -7641,10 +7611,10 @@
         <f>'Cohorte ficticio'!B57</f>
         <v>40-44</v>
       </c>
-      <c r="C18" s="57" t="n">
+      <c r="C18" s="58" t="n">
         <v>40</v>
       </c>
-      <c r="D18" s="58" t="n">
+      <c r="D18" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E18" s="42">
@@ -7659,36 +7629,35 @@
         <f>F18/E18</f>
         <v>0.00163510366982957</v>
       </c>
-      <c r="H18" s="59">
-        <f>D18/2</f>
+      <c r="H18" s="49">
+        <f>(2*D18*G18)/(2+D18*G18)</f>
+        <v>0.00814223485392217</v>
+      </c>
+      <c r="I18" s="49">
+        <f>1-H18</f>
+        <v>0.991857765146078</v>
+      </c>
+      <c r="J18" s="42">
+        <f>J17*I17</f>
+        <v>97052.5672980952</v>
+      </c>
+      <c r="K18" s="42">
+        <f>J18*H18</f>
+        <v>790.224796117178</v>
+      </c>
+      <c r="L18" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I18" s="49">
-        <f>D18*G18/(1+(D18-H18)*G18)</f>
-        <v>0.00814223485392217</v>
-      </c>
-      <c r="J18" s="49">
-        <f>1-I18</f>
-        <v>0.991857765146078</v>
-      </c>
-      <c r="K18" s="42">
-        <f>K17-L17</f>
-        <v>97055.1521133399</v>
-      </c>
-      <c r="L18" s="42">
-        <f>K18*I18</f>
-        <v>790.245842289955</v>
-      </c>
       <c r="M18" s="42">
-        <f>D18*K19+H18*L18</f>
-        <v>483300.145960975</v>
+        <f>J19*D18+K18*L18</f>
+        <v>483287.274500183</v>
       </c>
       <c r="N18" s="42">
         <f>SUM(M18:$M$25)</f>
-        <v>4454172.8128193</v>
-      </c>
-      <c r="O18" s="60">
-        <f>N18/K18</f>
+        <v>4454054.18734154</v>
+      </c>
+      <c r="O18" s="61">
+        <f>N18/J18</f>
         <v>45.8932134547352</v>
       </c>
       <c r="P18" s="29" t="n"/>
@@ -7717,36 +7686,35 @@
         <f>F19/E19</f>
         <v>0.00254255289732353</v>
       </c>
-      <c r="H19" s="50">
-        <f>D19/2</f>
+      <c r="H19" s="55">
+        <f>(2*D19*G19)/(2+D19*G19)</f>
+        <v>0.0126324676932829</v>
+      </c>
+      <c r="I19" s="55">
+        <f>1-H19</f>
+        <v>0.987367532306717</v>
+      </c>
+      <c r="J19" s="39">
+        <f>J18*I18</f>
+        <v>96262.342501978</v>
+      </c>
+      <c r="K19" s="39">
+        <f>J19*H19</f>
+        <v>1216.03093173597</v>
+      </c>
+      <c r="L19" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I19" s="55">
-        <f>D19*G19/(1+(D19-H19)*G19)</f>
-        <v>0.0126324676932829</v>
-      </c>
-      <c r="J19" s="55">
-        <f>1-I19</f>
-        <v>0.987367532306717</v>
-      </c>
-      <c r="K19" s="39">
-        <f>K18-L18</f>
-        <v>96264.90627105</v>
-      </c>
-      <c r="L19" s="39">
-        <f>K19*I19</f>
-        <v>1216.06331846594</v>
-      </c>
       <c r="M19" s="39">
-        <f>D19*K20+H19*L19</f>
-        <v>478284.373059085</v>
+        <f>J20*D19+K19*L19</f>
+        <v>478271.63518055</v>
       </c>
       <c r="N19" s="39">
         <f>SUM(M19:$M$25)</f>
-        <v>3970872.66685833</v>
-      </c>
-      <c r="O19" s="56">
-        <f>N19/K19</f>
+        <v>3970766.91284135</v>
+      </c>
+      <c r="O19" s="57">
+        <f>N19/J19</f>
         <v>41.2494316015607</v>
       </c>
       <c r="P19" s="29" t="n"/>
@@ -7757,10 +7725,10 @@
         <f>'Cohorte ficticio'!B59</f>
         <v>50-54</v>
       </c>
-      <c r="C20" s="57" t="n">
+      <c r="C20" s="58" t="n">
         <v>50</v>
       </c>
-      <c r="D20" s="58" t="n">
+      <c r="D20" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E20" s="42">
@@ -7775,36 +7743,35 @@
         <f>F20/E20</f>
         <v>0.00364174619463328</v>
       </c>
-      <c r="H20" s="59">
-        <f>D20/2</f>
+      <c r="H20" s="49">
+        <f>(2*D20*G20)/(2+D20*G20)</f>
+        <v>0.0180444477260648</v>
+      </c>
+      <c r="I20" s="49">
+        <f>1-H20</f>
+        <v>0.981955552273935</v>
+      </c>
+      <c r="J20" s="42">
+        <f>J19*I19</f>
+        <v>95046.311570242</v>
+      </c>
+      <c r="K20" s="42">
+        <f>J20*H20</f>
+        <v>1715.0582006845</v>
+      </c>
+      <c r="L20" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I20" s="49">
-        <f>D20*G20/(1+(D20-H20)*G20)</f>
-        <v>0.0180444477260648</v>
-      </c>
-      <c r="J20" s="49">
-        <f>1-I20</f>
-        <v>0.981955552273935</v>
-      </c>
-      <c r="K20" s="42">
-        <f>K19-L19</f>
-        <v>95048.8429525841</v>
-      </c>
-      <c r="L20" s="42">
-        <f>K20*I20</f>
-        <v>1715.10387808084</v>
-      </c>
       <c r="M20" s="42">
-        <f>D20*K21+H20*L20</f>
-        <v>470956.455067718</v>
+        <f>J21*D20+K20*L20</f>
+        <v>470943.912349499</v>
       </c>
       <c r="N20" s="42">
         <f>SUM(M20:$M$25)</f>
-        <v>3492588.29379924</v>
-      </c>
-      <c r="O20" s="60">
-        <f>N20/K20</f>
+        <v>3492495.2776608</v>
+      </c>
+      <c r="O20" s="61">
+        <f>N20/J20</f>
         <v>36.7451952628351</v>
       </c>
       <c r="P20" s="29" t="n"/>
@@ -7833,36 +7800,35 @@
         <f>F21/E21</f>
         <v>0.00574291010746076</v>
       </c>
-      <c r="H21" s="50">
-        <f>D21/2</f>
+      <c r="H21" s="55">
+        <f>(2*D21*G21)/(2+D21*G21)</f>
+        <v>0.0283081230227276</v>
+      </c>
+      <c r="I21" s="55">
+        <f>1-H21</f>
+        <v>0.971691876977272</v>
+      </c>
+      <c r="J21" s="39">
+        <f>J20*I20</f>
+        <v>93331.2533695575</v>
+      </c>
+      <c r="K21" s="39">
+        <f>J21*H21</f>
+        <v>2642.0326022508</v>
+      </c>
+      <c r="L21" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I21" s="55">
-        <f>D21*G21/(1+(D21-H21)*G21)</f>
-        <v>0.0283081230227276</v>
-      </c>
-      <c r="J21" s="55">
-        <f>1-I21</f>
-        <v>0.971691876977272</v>
-      </c>
-      <c r="K21" s="39">
-        <f>K20-L20</f>
-        <v>93333.7390745032</v>
-      </c>
-      <c r="L21" s="39">
-        <f>K21*I21</f>
-        <v>2642.1029678922</v>
-      </c>
       <c r="M21" s="39">
-        <f>D21*K22+H21*L21</f>
-        <v>460063.437952785</v>
+        <f>J22*D21+K21*L21</f>
+        <v>460051.185342161</v>
       </c>
       <c r="N21" s="39">
         <f>SUM(M21:$M$25)</f>
-        <v>3021631.83873153</v>
-      </c>
-      <c r="O21" s="56">
-        <f>N21/K21</f>
+        <v>3021551.3653113</v>
+      </c>
+      <c r="O21" s="57">
+        <f>N21/J21</f>
         <v>32.3744861043178</v>
       </c>
       <c r="P21" s="29" t="n"/>
@@ -7873,10 +7839,10 @@
         <f>'Cohorte ficticio'!B61</f>
         <v>60-64</v>
       </c>
-      <c r="C22" s="57" t="n">
+      <c r="C22" s="58" t="n">
         <v>60</v>
       </c>
-      <c r="D22" s="58" t="n">
+      <c r="D22" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E22" s="42">
@@ -7891,36 +7857,35 @@
         <f>F22/E22</f>
         <v>0.0082074428447314</v>
       </c>
-      <c r="H22" s="59">
-        <f>D22/2</f>
+      <c r="H22" s="49">
+        <f>(2*D22*G22)/(2+D22*G22)</f>
+        <v>0.0402121175818602</v>
+      </c>
+      <c r="I22" s="49">
+        <f>1-H22</f>
+        <v>0.95978788241814</v>
+      </c>
+      <c r="J22" s="42">
+        <f>J21*I21</f>
+        <v>90689.2207673068</v>
+      </c>
+      <c r="K22" s="42">
+        <f>J22*H22</f>
+        <v>3646.80560890222</v>
+      </c>
+      <c r="L22" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I22" s="49">
-        <f>D22*G22/(1+(D22-H22)*G22)</f>
-        <v>0.0402121175818602</v>
-      </c>
-      <c r="J22" s="49">
-        <f>1-I22</f>
-        <v>0.95978788241814</v>
-      </c>
-      <c r="K22" s="42">
-        <f>K21-L21</f>
-        <v>90691.636106611</v>
-      </c>
-      <c r="L22" s="42">
-        <f>K22*I22</f>
-        <v>3646.90273481032</v>
-      </c>
       <c r="M22" s="42">
-        <f>D22*K23+H22*L22</f>
-        <v>444340.923696029</v>
+        <f>J23*D22+K22*L22</f>
+        <v>444329.089814278</v>
       </c>
       <c r="N22" s="42">
         <f>SUM(M22:$M$25)</f>
-        <v>2561568.40077874</v>
-      </c>
-      <c r="O22" s="60">
-        <f>N22/K22</f>
+        <v>2561500.17996914</v>
+      </c>
+      <c r="O22" s="61">
+        <f>N22/J22</f>
         <v>28.2448140837104</v>
       </c>
       <c r="P22" s="29" t="n"/>
@@ -7949,36 +7914,35 @@
         <f>F23/E23</f>
         <v>0.0119798542647294</v>
       </c>
-      <c r="H23" s="50">
-        <f>D23/2</f>
+      <c r="H23" s="55">
+        <f>(2*D23*G23)/(2+D23*G23)</f>
+        <v>0.0581574761033407</v>
+      </c>
+      <c r="I23" s="55">
+        <f>1-H23</f>
+        <v>0.941842523896659</v>
+      </c>
+      <c r="J23" s="39">
+        <f>J22*I22</f>
+        <v>87042.4151584045</v>
+      </c>
+      <c r="K23" s="39">
+        <f>J23*H23</f>
+        <v>5062.16717955197</v>
+      </c>
+      <c r="L23" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I23" s="55">
-        <f>D23*G23/(1+(D23-H23)*G23)</f>
-        <v>0.0581574761033407</v>
-      </c>
-      <c r="J23" s="55">
-        <f>1-I23</f>
-        <v>0.941842523896659</v>
-      </c>
-      <c r="K23" s="39">
-        <f>K22-L22</f>
-        <v>87044.7333718007</v>
-      </c>
-      <c r="L23" s="39">
-        <f>K23*I23</f>
-        <v>5062.30200099216</v>
-      </c>
       <c r="M23" s="39">
-        <f>D23*K24+H23*L23</f>
-        <v>422567.911856523</v>
+        <f>J24*D23+K23*L23</f>
+        <v>422556.657843143</v>
       </c>
       <c r="N23" s="39">
         <f>SUM(M23:$M$25)</f>
-        <v>2117227.47708271</v>
-      </c>
-      <c r="O23" s="56">
-        <f>N23/K23</f>
+        <v>2117171.09015487</v>
+      </c>
+      <c r="O23" s="57">
+        <f>N23/J23</f>
         <v>24.3234414658867</v>
       </c>
       <c r="P23" s="29" t="n"/>
@@ -7989,10 +7953,10 @@
         <f>'Cohorte ficticio'!B63</f>
         <v>70-74</v>
       </c>
-      <c r="C24" s="57" t="n">
+      <c r="C24" s="58" t="n">
         <v>70</v>
       </c>
-      <c r="D24" s="58" t="n">
+      <c r="D24" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E24" s="42">
@@ -8007,37 +7971,36 @@
         <f>F24/E24</f>
         <v>0.0192046463689099</v>
       </c>
-      <c r="H24" s="59">
-        <f>D24/2</f>
+      <c r="H24" s="49">
+        <f>(2*D24*G24)/(2+D24*G24)</f>
+        <v>0.0916242056726126</v>
+      </c>
+      <c r="I24" s="49">
+        <f>1-H24</f>
+        <v>0.908375794327388</v>
+      </c>
+      <c r="J24" s="42">
+        <f>J23*I23</f>
+        <v>81980.2479788526</v>
+      </c>
+      <c r="K24" s="42">
+        <f>J24*H24</f>
+        <v>7511.37510190617</v>
+      </c>
+      <c r="L24" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I24" s="49">
-        <f>D24*G24/(1+(D24-H24)*G24)</f>
-        <v>0.0916242056726126</v>
-      </c>
-      <c r="J24" s="49">
-        <f>1-I24</f>
-        <v>0.908375794327388</v>
-      </c>
-      <c r="K24" s="42">
-        <f>K23-L23</f>
-        <v>81982.4313708085</v>
-      </c>
-      <c r="L24" s="42">
-        <f>K24*I24</f>
-        <v>7511.5751534598</v>
-      </c>
       <c r="M24" s="42">
-        <f>D24*K25+H24*L24</f>
-        <v>391133.218970393</v>
+        <f>J25*D24+K24*L24</f>
+        <v>391122.802139497</v>
       </c>
       <c r="N24" s="42">
         <f>SUM(M24:$M$25)</f>
-        <v>1694659.56522619</v>
-      </c>
-      <c r="O24" s="60">
-        <f>N24/K24</f>
-        <v>20.6710088599495</v>
+        <v>1694614.43231172</v>
+      </c>
+      <c r="O24" s="61">
+        <f>N24/J24</f>
+        <v>20.6710088599496</v>
       </c>
       <c r="P24" s="29" t="n"/>
     </row>
@@ -8067,36 +8030,35 @@
         <f>F25/E25</f>
         <v>0.0571303038341007</v>
       </c>
-      <c r="H25" s="61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I25" s="55" t="n">
+      <c r="H25" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="J25" s="55">
-        <f>1-I25</f>
+      <c r="I25" s="55">
+        <f>1-H25</f>
         <v>0</v>
       </c>
+      <c r="J25" s="39">
+        <f>J24*I24</f>
+        <v>74468.8728769464</v>
+      </c>
       <c r="K25" s="39">
-        <f>K24-L24</f>
-        <v>74470.8562173487</v>
-      </c>
-      <c r="L25" s="39">
-        <f>K25*I25</f>
-        <v>74470.8562173487</v>
+        <f>J25*H25</f>
+        <v>74468.8728769464</v>
+      </c>
+      <c r="L25" s="56">
+        <f>1/G25</f>
+        <v>17.5038452955524</v>
       </c>
       <c r="M25" s="39">
-        <f>K25/G25</f>
-        <v>1303526.3462558</v>
+        <f>K25*L25</f>
+        <v>1303491.63017222</v>
       </c>
       <c r="N25" s="39">
         <f>SUM(M25:$M$25)</f>
-        <v>1303526.3462558</v>
-      </c>
-      <c r="O25" s="56">
-        <f>N25/K25</f>
+        <v>1303491.63017222</v>
+      </c>
+      <c r="O25" s="57">
+        <f>N25/J25</f>
         <v>17.5038452955524</v>
       </c>
       <c r="P25" s="29" t="n"/>
@@ -8127,7 +8089,7 @@
         </is>
       </c>
       <c r="E27" s="48">
-        <f>ROUND(SUM(L9:L25)-D5,6)</f>
+        <f>ROUND(SUM(K9:K25)-D5,6)</f>
         <v>0</v>
       </c>
       <c r="F27" s="35" t="inlineStr">
@@ -8148,12 +8110,12 @@
       <c r="A28" s="29" t="n"/>
       <c r="B28" s="62" t="inlineStr">
         <is>
-          <t>q0 (mortalidad infantil, por mil)</t>
-        </is>
-      </c>
-      <c r="E28" s="56">
-        <f>I9*1000</f>
-        <v>7.81956520783196</v>
+          <t>q0 (por mil)</t>
+        </is>
+      </c>
+      <c r="E28" s="57">
+        <f>H9*1000</f>
+        <v>7.84563539639034</v>
       </c>
       <c r="F28" s="29" t="n"/>
       <c r="G28" s="29" t="n"/>
@@ -8267,11 +8229,11 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="9" customWidth="1" min="15" max="15"/>
@@ -8387,7 +8349,7 @@
       <c r="A6" s="29" t="n"/>
       <c r="B6" s="35" t="inlineStr">
         <is>
-          <t>nMx = D/P;  nqx = n·nMx / (1 + (n − nax)·nMx);  lx+n = lx·(1 − nqx);  ndx = lx − lx+n;  nLx = n·lx+n + nax·ndx;  Tx = suma de nLx hacia abajo;  ex = Tx/lx.  Grupo abierto 75+: q = 1 y L = l/M.</t>
+          <t>nmx = D/P;  nqx = (2·n·nmx) / (2 + n·nmx);  npx = 1 − nqx;  lx+n = lx·npx;  ndx = lx·nqx;  nLx = lx+n·n + ndx·nAx;  Tx = suma de nLx hacia abajo;  ex = Tx/lx.</t>
         </is>
       </c>
       <c r="P6" s="29" t="n"/>
@@ -8396,7 +8358,7 @@
       <c r="A7" s="29" t="n"/>
       <c r="B7" s="35" t="inlineStr">
         <is>
-          <t>nax: para 0 y 1-4, Coale-Demeny según la mortalidad infantil y el sexo (en ambos sexos, el promedio de hombres y mujeres); n/2 en los demás grupos. Valores sin redondear.</t>
+          <t>nAx: 0.12 en la edad 0, 1.5 en 1-4 y 2.5 en los demás grupos (los valores del Cuadro 4.3 del ejemplo de la profesora). En el grupo abierto 75+: nqx = 1 y nAx = 1/nmx.</t>
         </is>
       </c>
       <c r="P7" s="29" t="n"/>
@@ -8430,32 +8392,32 @@
       </c>
       <c r="G8" s="37" t="inlineStr">
         <is>
-          <t>nMx</t>
+          <t>nmx</t>
         </is>
       </c>
       <c r="H8" s="37" t="inlineStr">
         <is>
-          <t>nax</t>
+          <t>nqx</t>
         </is>
       </c>
       <c r="I8" s="37" t="inlineStr">
         <is>
-          <t>nqx</t>
+          <t>npx</t>
         </is>
       </c>
       <c r="J8" s="37" t="inlineStr">
         <is>
-          <t>npx</t>
+          <t>lx</t>
         </is>
       </c>
       <c r="K8" s="37" t="inlineStr">
         <is>
-          <t>lx</t>
+          <t>ndx</t>
         </is>
       </c>
       <c r="L8" s="37" t="inlineStr">
         <is>
-          <t>ndx</t>
+          <t>nAx</t>
         </is>
       </c>
       <c r="M8" s="37" t="inlineStr">
@@ -8499,37 +8461,36 @@
         <f>F9/E9</f>
         <v>0.00896196636663077</v>
       </c>
-      <c r="H9" s="50">
-        <f>(IF($G$9&gt;=0.107,0.33,0.045+2.684*$G$9)+IF($G$9&gt;=0.107,0.35,0.053+2.8*$G$9))/2</f>
-        <v>0.0735737117773016</v>
+      <c r="H9" s="55">
+        <f>(2*D9*G9)/(2+D9*G9)</f>
+        <v>0.00892198709250748</v>
       </c>
       <c r="I9" s="55">
-        <f>D9*G9/(1+(D9-H9)*G9)</f>
-        <v>0.00888817142358165</v>
-      </c>
-      <c r="J9" s="55">
-        <f>1-I9</f>
-        <v>0.991111828576418</v>
-      </c>
-      <c r="K9" s="39">
+        <f>1-H9</f>
+        <v>0.991078012907493</v>
+      </c>
+      <c r="J9" s="39">
         <f>$D$5</f>
         <v>100000</v>
       </c>
-      <c r="L9" s="39">
-        <f>K9*I9</f>
-        <v>888.817142358165</v>
+      <c r="K9" s="39">
+        <f>J9*H9</f>
+        <v>892.198709250748</v>
+      </c>
+      <c r="L9" s="56" t="n">
+        <v>0.12</v>
       </c>
       <c r="M9" s="39">
-        <f>D9*K10+H9*L9</f>
-        <v>99176.5764338964</v>
+        <f>J10*D9+K9*L9</f>
+        <v>99214.8651358594</v>
       </c>
       <c r="N9" s="39">
         <f>SUM(M9:$M$25)</f>
-        <v>8030941.40615</v>
-      </c>
-      <c r="O9" s="56">
-        <f>N9/K9</f>
-        <v>80.3094140615</v>
+        <v>8030694.10568805</v>
+      </c>
+      <c r="O9" s="57">
+        <f>N9/J9</f>
+        <v>80.3069410568805</v>
       </c>
       <c r="P9" s="29" t="n"/>
     </row>
@@ -8539,10 +8500,10 @@
         <f>'Cohorte ficticio'!B49</f>
         <v>1-4</v>
       </c>
-      <c r="C10" s="57" t="n">
+      <c r="C10" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="58" t="n">
+      <c r="D10" s="59" t="n">
         <v>4</v>
       </c>
       <c r="E10" s="42">
@@ -8557,37 +8518,36 @@
         <f>F10/E10</f>
         <v>0.000457321347939266</v>
       </c>
-      <c r="H10" s="59">
-        <f>(IF($G$9&gt;=0.107,1.352,1.651-2.816*$G$9)+IF($G$9&gt;=0.107,1.361,1.522-1.518*$G$9))/2</f>
-        <v>1.56707941888351</v>
+      <c r="H10" s="49">
+        <f>(2*D10*G10)/(2+D10*G10)</f>
+        <v>0.00182761377816398</v>
       </c>
       <c r="I10" s="49">
-        <f>D10*G10/(1+(D10-H10)*G10)</f>
-        <v>0.001827252342343</v>
-      </c>
-      <c r="J10" s="49">
-        <f>1-I10</f>
-        <v>0.998172747657657</v>
+        <f>1-H10</f>
+        <v>0.998172386221836</v>
+      </c>
+      <c r="J10" s="42">
+        <f>J9*I9</f>
+        <v>99107.8012907493</v>
       </c>
       <c r="K10" s="42">
-        <f>K9-L9</f>
-        <v>99111.1828576418</v>
-      </c>
-      <c r="L10" s="42">
-        <f>K10*I10</f>
-        <v>181.101141029011</v>
+        <f>J10*H10</f>
+        <v>181.130783162511</v>
+      </c>
+      <c r="L10" s="60" t="n">
+        <v>1.5</v>
       </c>
       <c r="M10" s="42">
-        <f>D10*K11+H10*L10</f>
-        <v>396004.126737294</v>
+        <f>J11*D10+K10*L10</f>
+        <v>395978.378205091</v>
       </c>
       <c r="N10" s="42">
         <f>SUM(M10:$M$25)</f>
-        <v>7931764.8297161</v>
-      </c>
-      <c r="O10" s="60">
-        <f>N10/K10</f>
-        <v>80.0289594072233</v>
+        <v>7931479.24055219</v>
+      </c>
+      <c r="O10" s="61">
+        <f>N10/J10</f>
+        <v>80.0288084011053</v>
       </c>
       <c r="P10" s="29" t="n"/>
     </row>
@@ -8615,36 +8575,35 @@
         <f>F11/E11</f>
         <v>0.000199409726685929</v>
       </c>
-      <c r="H11" s="50">
-        <f>D11/2</f>
+      <c r="H11" s="55">
+        <f>(2*D11*G11)/(2+D11*G11)</f>
+        <v>0.000996551828110468</v>
+      </c>
+      <c r="I11" s="55">
+        <f>1-H11</f>
+        <v>0.99900344817189</v>
+      </c>
+      <c r="J11" s="39">
+        <f>J10*I10</f>
+        <v>98926.6705075867</v>
+      </c>
+      <c r="K11" s="39">
+        <f>J11*H11</f>
+        <v>98.5855543432175</v>
+      </c>
+      <c r="L11" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I11" s="55">
-        <f>D11*G11/(1+(D11-H11)*G11)</f>
-        <v>0.000996551828110468</v>
-      </c>
-      <c r="J11" s="55">
-        <f>1-I11</f>
-        <v>0.99900344817189</v>
-      </c>
-      <c r="K11" s="39">
-        <f>K10-L10</f>
-        <v>98930.0817166128</v>
-      </c>
-      <c r="L11" s="39">
-        <f>K11*I11</f>
-        <v>98.5889537898085</v>
-      </c>
       <c r="M11" s="39">
-        <f>D11*K12+H11*L11</f>
-        <v>494403.93619859</v>
+        <f>J12*D11+K11*L11</f>
+        <v>494386.888652076</v>
       </c>
       <c r="N11" s="39">
         <f>SUM(M11:$M$25)</f>
-        <v>7535760.70297881</v>
-      </c>
-      <c r="O11" s="56">
-        <f>N11/K11</f>
+        <v>7535500.86234709</v>
+      </c>
+      <c r="O11" s="57">
+        <f>N11/J11</f>
         <v>76.1725915133189</v>
       </c>
       <c r="P11" s="29" t="n"/>
@@ -8655,10 +8614,10 @@
         <f>'Cohorte ficticio'!B51</f>
         <v>10-14</v>
       </c>
-      <c r="C12" s="57" t="n">
+      <c r="C12" s="58" t="n">
         <v>10</v>
       </c>
-      <c r="D12" s="58" t="n">
+      <c r="D12" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E12" s="42">
@@ -8673,36 +8632,35 @@
         <f>F12/E12</f>
         <v>0.000281330419259546</v>
       </c>
-      <c r="H12" s="59">
-        <f>D12/2</f>
+      <c r="H12" s="49">
+        <f>(2*D12*G12)/(2+D12*G12)</f>
+        <v>0.00140566345657379</v>
+      </c>
+      <c r="I12" s="49">
+        <f>1-H12</f>
+        <v>0.998594336543426</v>
+      </c>
+      <c r="J12" s="42">
+        <f>J11*I11</f>
+        <v>98828.0849532435</v>
+      </c>
+      <c r="K12" s="42">
+        <f>J12*H12</f>
+        <v>138.919027501945</v>
+      </c>
+      <c r="L12" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I12" s="49">
-        <f>D12*G12/(1+(D12-H12)*G12)</f>
-        <v>0.00140566345657379</v>
-      </c>
-      <c r="J12" s="49">
-        <f>1-I12</f>
-        <v>0.998594336543426</v>
-      </c>
-      <c r="K12" s="42">
-        <f>K11-L11</f>
-        <v>98831.492762823</v>
-      </c>
-      <c r="L12" s="42">
-        <f>K12*I12</f>
-        <v>138.923817735337</v>
-      </c>
       <c r="M12" s="42">
-        <f>D12*K13+H12*L12</f>
-        <v>493810.154269777</v>
+        <f>J13*D12+K12*L12</f>
+        <v>493793.127197463</v>
       </c>
       <c r="N12" s="42">
         <f>SUM(M12:$M$25)</f>
-        <v>7041356.76678021</v>
-      </c>
-      <c r="O12" s="60">
-        <f>N12/K12</f>
+        <v>7041113.97369502</v>
+      </c>
+      <c r="O12" s="61">
+        <f>N12/J12</f>
         <v>71.2460833074549</v>
       </c>
       <c r="P12" s="29" t="n"/>
@@ -8731,36 +8689,35 @@
         <f>F13/E13</f>
         <v>0.000828525352993602</v>
       </c>
-      <c r="H13" s="50">
-        <f>D13/2</f>
+      <c r="H13" s="55">
+        <f>(2*D13*G13)/(2+D13*G13)</f>
+        <v>0.00413406382324688</v>
+      </c>
+      <c r="I13" s="55">
+        <f>1-H13</f>
+        <v>0.995865936176753</v>
+      </c>
+      <c r="J13" s="39">
+        <f>J12*I12</f>
+        <v>98689.1659257416</v>
+      </c>
+      <c r="K13" s="39">
+        <f>J13*H13</f>
+        <v>407.987310600017</v>
+      </c>
+      <c r="L13" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I13" s="55">
-        <f>D13*G13/(1+(D13-H13)*G13)</f>
-        <v>0.00413406382324688</v>
-      </c>
-      <c r="J13" s="55">
-        <f>1-I13</f>
-        <v>0.995865936176753</v>
-      </c>
-      <c r="K13" s="39">
-        <f>K12-L12</f>
-        <v>98692.5689450877</v>
-      </c>
-      <c r="L13" s="39">
-        <f>K13*I13</f>
-        <v>408.001378899185</v>
-      </c>
       <c r="M13" s="39">
-        <f>D13*K14+H13*L13</f>
-        <v>492442.841278191</v>
+        <f>J14*D13+K13*L13</f>
+        <v>492425.861352208</v>
       </c>
       <c r="N13" s="39">
         <f>SUM(M13:$M$25)</f>
-        <v>6547546.61251044</v>
-      </c>
-      <c r="O13" s="56">
-        <f>N13/K13</f>
+        <v>6547320.84649756</v>
+      </c>
+      <c r="O13" s="57">
+        <f>N13/J13</f>
         <v>66.342853190431</v>
       </c>
       <c r="P13" s="29" t="n"/>
@@ -8771,10 +8728,10 @@
         <f>'Cohorte ficticio'!B53</f>
         <v>20-24</v>
       </c>
-      <c r="C14" s="57" t="n">
+      <c r="C14" s="58" t="n">
         <v>20</v>
       </c>
-      <c r="D14" s="58" t="n">
+      <c r="D14" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E14" s="42">
@@ -8789,36 +8746,35 @@
         <f>F14/E14</f>
         <v>0.0012679045315357</v>
       </c>
-      <c r="H14" s="59">
-        <f>D14/2</f>
+      <c r="H14" s="49">
+        <f>(2*D14*G14)/(2+D14*G14)</f>
+        <v>0.00631949137828968</v>
+      </c>
+      <c r="I14" s="49">
+        <f>1-H14</f>
+        <v>0.99368050862171</v>
+      </c>
+      <c r="J14" s="42">
+        <f>J13*I13</f>
+        <v>98281.1786151416</v>
+      </c>
+      <c r="K14" s="42">
+        <f>J14*H14</f>
+        <v>621.087060906535</v>
+      </c>
+      <c r="L14" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I14" s="49">
-        <f>D14*G14/(1+(D14-H14)*G14)</f>
-        <v>0.00631949137828968</v>
-      </c>
-      <c r="J14" s="49">
-        <f>1-I14</f>
-        <v>0.99368050862171</v>
-      </c>
-      <c r="K14" s="42">
-        <f>K13-L13</f>
-        <v>98284.5675661885</v>
-      </c>
-      <c r="L14" s="42">
-        <f>K14*I14</f>
-        <v>621.108477353458</v>
-      </c>
       <c r="M14" s="42">
-        <f>D14*K15+H14*L14</f>
-        <v>489870.066637559</v>
+        <f>J15*D14+K14*L14</f>
+        <v>489853.175423441</v>
       </c>
       <c r="N14" s="42">
         <f>SUM(M14:$M$25)</f>
-        <v>6055103.77123225</v>
-      </c>
-      <c r="O14" s="60">
-        <f>N14/K14</f>
+        <v>6054894.98514535</v>
+      </c>
+      <c r="O14" s="61">
+        <f>N14/J14</f>
         <v>61.6078792548435</v>
       </c>
       <c r="P14" s="29" t="n"/>
@@ -8847,36 +8803,35 @@
         <f>F15/E15</f>
         <v>0.0015673240507028</v>
       </c>
-      <c r="H15" s="50">
-        <f>D15/2</f>
+      <c r="H15" s="55">
+        <f>(2*D15*G15)/(2+D15*G15)</f>
+        <v>0.00780603379225599</v>
+      </c>
+      <c r="I15" s="55">
+        <f>1-H15</f>
+        <v>0.992193966207744</v>
+      </c>
+      <c r="J15" s="39">
+        <f>J14*I14</f>
+        <v>97660.091554235</v>
+      </c>
+      <c r="K15" s="39">
+        <f>J15*H15</f>
+        <v>762.337974827172</v>
+      </c>
+      <c r="L15" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I15" s="55">
-        <f>D15*G15/(1+(D15-H15)*G15)</f>
-        <v>0.00780603379225599</v>
-      </c>
-      <c r="J15" s="55">
-        <f>1-I15</f>
-        <v>0.992193966207744</v>
-      </c>
-      <c r="K15" s="39">
-        <f>K14-L14</f>
-        <v>97663.4590888351</v>
-      </c>
-      <c r="L15" s="39">
-        <f>K15*I15</f>
-        <v>762.364261916056</v>
-      </c>
       <c r="M15" s="39">
-        <f>D15*K16+H15*L15</f>
-        <v>486411.384789385</v>
+        <f>J16*D15+K15*L15</f>
+        <v>486394.612834107</v>
       </c>
       <c r="N15" s="39">
         <f>SUM(M15:$M$25)</f>
-        <v>5565233.70459469</v>
-      </c>
-      <c r="O15" s="56">
-        <f>N15/K15</f>
+        <v>5565041.80972191</v>
+      </c>
+      <c r="O15" s="57">
+        <f>N15/J15</f>
         <v>56.983786530974</v>
       </c>
       <c r="P15" s="29" t="n"/>
@@ -8887,10 +8842,10 @@
         <f>'Cohorte ficticio'!B55</f>
         <v>30-34</v>
       </c>
-      <c r="C16" s="57" t="n">
+      <c r="C16" s="58" t="n">
         <v>30</v>
       </c>
-      <c r="D16" s="58" t="n">
+      <c r="D16" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E16" s="42">
@@ -8905,36 +8860,35 @@
         <f>F16/E16</f>
         <v>0.0018528230870593</v>
       </c>
-      <c r="H16" s="59">
-        <f>D16/2</f>
+      <c r="H16" s="49">
+        <f>(2*D16*G16)/(2+D16*G16)</f>
+        <v>0.00922140137190424</v>
+      </c>
+      <c r="I16" s="49">
+        <f>1-H16</f>
+        <v>0.990778598628096</v>
+      </c>
+      <c r="J16" s="42">
+        <f>J15*I15</f>
+        <v>96897.7535794079</v>
+      </c>
+      <c r="K16" s="42">
+        <f>J16*H16</f>
+        <v>893.53307779159</v>
+      </c>
+      <c r="L16" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I16" s="49">
-        <f>D16*G16/(1+(D16-H16)*G16)</f>
-        <v>0.00922140137190424</v>
-      </c>
-      <c r="J16" s="49">
-        <f>1-I16</f>
-        <v>0.990778598628096</v>
-      </c>
-      <c r="K16" s="42">
-        <f>K15-L15</f>
-        <v>96901.094826919</v>
-      </c>
-      <c r="L16" s="42">
-        <f>K16*I16</f>
-        <v>893.563888775973</v>
-      </c>
       <c r="M16" s="42">
-        <f>D16*K17+H16*L16</f>
-        <v>482271.564412655</v>
+        <f>J17*D16+K16*L16</f>
+        <v>482254.93520256</v>
       </c>
       <c r="N16" s="42">
         <f>SUM(M16:$M$25)</f>
-        <v>5078822.3198053</v>
-      </c>
-      <c r="O16" s="60">
-        <f>N16/K16</f>
+        <v>5078647.1968878</v>
+      </c>
+      <c r="O16" s="61">
+        <f>N16/J16</f>
         <v>52.412434853052</v>
       </c>
       <c r="P16" s="29" t="n"/>
@@ -8963,36 +8917,35 @@
         <f>F17/E17</f>
         <v>0.00216434937169194</v>
       </c>
-      <c r="H17" s="50">
-        <f>D17/2</f>
+      <c r="H17" s="55">
+        <f>(2*D17*G17)/(2+D17*G17)</f>
+        <v>0.01076350688505</v>
+      </c>
+      <c r="I17" s="55">
+        <f>1-H17</f>
+        <v>0.98923649311495</v>
+      </c>
+      <c r="J17" s="39">
+        <f>J16*I16</f>
+        <v>96004.2205016163</v>
+      </c>
+      <c r="K17" s="39">
+        <f>J17*H17</f>
+        <v>1033.34208836301</v>
+      </c>
+      <c r="L17" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I17" s="55">
-        <f>D17*G17/(1+(D17-H17)*G17)</f>
-        <v>0.01076350688505</v>
-      </c>
-      <c r="J17" s="55">
-        <f>1-I17</f>
-        <v>0.98923649311495</v>
-      </c>
-      <c r="K17" s="39">
-        <f>K16-L16</f>
-        <v>96007.530938143</v>
-      </c>
-      <c r="L17" s="39">
-        <f>K17*I17</f>
-        <v>1033.37772026936</v>
-      </c>
       <c r="M17" s="39">
-        <f>D17*K18+H17*L17</f>
-        <v>477454.210390042</v>
+        <f>J18*D17+K17*L17</f>
+        <v>477437.747287174</v>
       </c>
       <c r="N17" s="39">
         <f>SUM(M17:$M$25)</f>
-        <v>4596550.75539265</v>
-      </c>
-      <c r="O17" s="56">
-        <f>N17/K17</f>
+        <v>4596392.26168524</v>
+      </c>
+      <c r="O17" s="57">
+        <f>N17/J17</f>
         <v>47.8769812167566</v>
       </c>
       <c r="P17" s="29" t="n"/>
@@ -9003,10 +8956,10 @@
         <f>'Cohorte ficticio'!B57</f>
         <v>40-44</v>
       </c>
-      <c r="C18" s="57" t="n">
+      <c r="C18" s="58" t="n">
         <v>40</v>
       </c>
-      <c r="D18" s="58" t="n">
+      <c r="D18" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E18" s="42">
@@ -9021,36 +8974,35 @@
         <f>F18/E18</f>
         <v>0.00273827709659221</v>
       </c>
-      <c r="H18" s="59">
-        <f>D18/2</f>
+      <c r="H18" s="49">
+        <f>(2*D18*G18)/(2+D18*G18)</f>
+        <v>0.0135982957285953</v>
+      </c>
+      <c r="I18" s="49">
+        <f>1-H18</f>
+        <v>0.986401704271405</v>
+      </c>
+      <c r="J18" s="42">
+        <f>J17*I17</f>
+        <v>94970.8784132533</v>
+      </c>
+      <c r="K18" s="42">
+        <f>J18*H18</f>
+        <v>1291.44209026789</v>
+      </c>
+      <c r="L18" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I18" s="49">
-        <f>D18*G18/(1+(D18-H18)*G18)</f>
-        <v>0.0135982957285953</v>
-      </c>
-      <c r="J18" s="49">
-        <f>1-I18</f>
-        <v>0.986401704271405</v>
-      </c>
-      <c r="K18" s="42">
-        <f>K17-L17</f>
-        <v>94974.1532178737</v>
-      </c>
-      <c r="L18" s="42">
-        <f>K18*I18</f>
-        <v>1291.48662202957</v>
-      </c>
       <c r="M18" s="42">
-        <f>D18*K19+H18*L18</f>
-        <v>471642.049534294</v>
+        <f>J19*D18+K18*L18</f>
+        <v>471625.786840597</v>
       </c>
       <c r="N18" s="42">
         <f>SUM(M18:$M$25)</f>
-        <v>4119096.54500261</v>
-      </c>
-      <c r="O18" s="60">
-        <f>N18/K18</f>
+        <v>4118954.51439807</v>
+      </c>
+      <c r="O18" s="61">
+        <f>N18/J18</f>
         <v>43.3707109296702</v>
       </c>
       <c r="P18" s="29" t="n"/>
@@ -9079,36 +9031,35 @@
         <f>F19/E19</f>
         <v>0.00386574757502374</v>
       </c>
-      <c r="H19" s="50">
-        <f>D19/2</f>
+      <c r="H19" s="55">
+        <f>(2*D19*G19)/(2+D19*G19)</f>
+        <v>0.0191437258457063</v>
+      </c>
+      <c r="I19" s="55">
+        <f>1-H19</f>
+        <v>0.980856274154294</v>
+      </c>
+      <c r="J19" s="39">
+        <f>J18*I18</f>
+        <v>93679.4363229854</v>
+      </c>
+      <c r="K19" s="39">
+        <f>J19*H19</f>
+        <v>1793.37344634753</v>
+      </c>
+      <c r="L19" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I19" s="55">
-        <f>D19*G19/(1+(D19-H19)*G19)</f>
-        <v>0.0191437258457063</v>
-      </c>
-      <c r="J19" s="55">
-        <f>1-I19</f>
-        <v>0.980856274154294</v>
-      </c>
-      <c r="K19" s="39">
-        <f>K18-L18</f>
-        <v>93682.6665958441</v>
-      </c>
-      <c r="L19" s="39">
-        <f>K19*I19</f>
-        <v>1793.43528580555</v>
-      </c>
       <c r="M19" s="39">
-        <f>D19*K20+H19*L19</f>
-        <v>463929.744764707</v>
+        <f>J20*D19+K19*L19</f>
+        <v>463913.747999058</v>
       </c>
       <c r="N19" s="39">
         <f>SUM(M19:$M$25)</f>
-        <v>3647454.49546831</v>
-      </c>
-      <c r="O19" s="56">
-        <f>N19/K19</f>
+        <v>3647328.72755747</v>
+      </c>
+      <c r="O19" s="57">
+        <f>N19/J19</f>
         <v>38.9341446823218</v>
       </c>
       <c r="P19" s="29" t="n"/>
@@ -9119,10 +9070,10 @@
         <f>'Cohorte ficticio'!B59</f>
         <v>50-54</v>
       </c>
-      <c r="C20" s="57" t="n">
+      <c r="C20" s="58" t="n">
         <v>50</v>
       </c>
-      <c r="D20" s="58" t="n">
+      <c r="D20" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E20" s="42">
@@ -9137,36 +9088,35 @@
         <f>F20/E20</f>
         <v>0.00520683622724415</v>
       </c>
-      <c r="H20" s="59">
-        <f>D20/2</f>
+      <c r="H20" s="49">
+        <f>(2*D20*G20)/(2+D20*G20)</f>
+        <v>0.0256996465100312</v>
+      </c>
+      <c r="I20" s="49">
+        <f>1-H20</f>
+        <v>0.974300353489969</v>
+      </c>
+      <c r="J20" s="42">
+        <f>J19*I19</f>
+        <v>91886.0628766379</v>
+      </c>
+      <c r="K20" s="42">
+        <f>J20*H20</f>
+        <v>2361.4393351281</v>
+      </c>
+      <c r="L20" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I20" s="49">
-        <f>D20*G20/(1+(D20-H20)*G20)</f>
-        <v>0.0256996465100312</v>
-      </c>
-      <c r="J20" s="49">
-        <f>1-I20</f>
-        <v>0.974300353489969</v>
-      </c>
-      <c r="K20" s="42">
-        <f>K19-L19</f>
-        <v>91889.2313100386</v>
-      </c>
-      <c r="L20" s="42">
-        <f>K20*I20</f>
-        <v>2361.52076274649</v>
-      </c>
       <c r="M20" s="42">
-        <f>D20*K21+H20*L20</f>
-        <v>453542.354643327</v>
+        <f>J21*D20+K20*L20</f>
+        <v>453526.716045369</v>
       </c>
       <c r="N20" s="42">
         <f>SUM(M20:$M$25)</f>
-        <v>3183524.75070361</v>
-      </c>
-      <c r="O20" s="60">
-        <f>N20/K20</f>
+        <v>3183414.97955841</v>
+      </c>
+      <c r="O20" s="61">
+        <f>N20/J20</f>
         <v>34.6452430313868</v>
       </c>
       <c r="P20" s="29" t="n"/>
@@ -9195,36 +9145,35 @@
         <f>F21/E21</f>
         <v>0.00770614020985947</v>
       </c>
-      <c r="H21" s="50">
-        <f>D21/2</f>
+      <c r="H21" s="55">
+        <f>(2*D21*G21)/(2+D21*G21)</f>
+        <v>0.037802424098361</v>
+      </c>
+      <c r="I21" s="55">
+        <f>1-H21</f>
+        <v>0.962197575901639</v>
+      </c>
+      <c r="J21" s="39">
+        <f>J20*I20</f>
+        <v>89524.6235415098</v>
+      </c>
+      <c r="K21" s="39">
+        <f>J21*H21</f>
+        <v>3384.24778636227</v>
+      </c>
+      <c r="L21" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I21" s="55">
-        <f>D21*G21/(1+(D21-H21)*G21)</f>
-        <v>0.037802424098361</v>
-      </c>
-      <c r="J21" s="55">
-        <f>1-I21</f>
-        <v>0.962197575901639</v>
-      </c>
-      <c r="K21" s="39">
-        <f>K20-L20</f>
-        <v>89527.7105472921</v>
-      </c>
-      <c r="L21" s="39">
-        <f>K21*I21</f>
-        <v>3384.36448266404</v>
-      </c>
       <c r="M21" s="39">
-        <f>D21*K22+H21*L21</f>
-        <v>439177.6415298</v>
+        <f>J22*D21+K21*L21</f>
+        <v>439162.498241643</v>
       </c>
       <c r="N21" s="39">
         <f>SUM(M21:$M$25)</f>
-        <v>2729982.39606028</v>
-      </c>
-      <c r="O21" s="56">
-        <f>N21/K21</f>
+        <v>2729888.26351304</v>
+      </c>
+      <c r="O21" s="57">
+        <f>N21/J21</f>
         <v>30.4931554640638</v>
       </c>
       <c r="P21" s="29" t="n"/>
@@ -9235,10 +9184,10 @@
         <f>'Cohorte ficticio'!B61</f>
         <v>60-64</v>
       </c>
-      <c r="C22" s="57" t="n">
+      <c r="C22" s="58" t="n">
         <v>60</v>
       </c>
-      <c r="D22" s="58" t="n">
+      <c r="D22" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E22" s="42">
@@ -9253,36 +9202,35 @@
         <f>F22/E22</f>
         <v>0.0106317004824762</v>
       </c>
-      <c r="H22" s="59">
-        <f>D22/2</f>
+      <c r="H22" s="49">
+        <f>(2*D22*G22)/(2+D22*G22)</f>
+        <v>0.0517821710792632</v>
+      </c>
+      <c r="I22" s="49">
+        <f>1-H22</f>
+        <v>0.948217828920737</v>
+      </c>
+      <c r="J22" s="42">
+        <f>J21*I21</f>
+        <v>86140.3757551475</v>
+      </c>
+      <c r="K22" s="42">
+        <f>J22*H22</f>
+        <v>4460.53567418506</v>
+      </c>
+      <c r="L22" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I22" s="49">
-        <f>D22*G22/(1+(D22-H22)*G22)</f>
-        <v>0.0517821710792632</v>
-      </c>
-      <c r="J22" s="49">
-        <f>1-I22</f>
-        <v>0.948217828920737</v>
-      </c>
-      <c r="K22" s="42">
-        <f>K21-L21</f>
-        <v>86143.346064628</v>
-      </c>
-      <c r="L22" s="42">
-        <f>K22*I22</f>
-        <v>4460.68948325874</v>
-      </c>
       <c r="M22" s="42">
-        <f>D22*K23+H22*L22</f>
-        <v>419565.006614993</v>
+        <f>J23*D22+K22*L22</f>
+        <v>419550.539590275</v>
       </c>
       <c r="N22" s="42">
         <f>SUM(M22:$M$25)</f>
-        <v>2290804.75453048</v>
-      </c>
-      <c r="O22" s="60">
-        <f>N22/K22</f>
+        <v>2290725.7652714</v>
+      </c>
+      <c r="O22" s="61">
+        <f>N22/J22</f>
         <v>26.5929390856472</v>
       </c>
       <c r="P22" s="29" t="n"/>
@@ -9311,36 +9259,35 @@
         <f>F23/E23</f>
         <v>0.0149094374061321</v>
       </c>
-      <c r="H23" s="50">
-        <f>D23/2</f>
+      <c r="H23" s="55">
+        <f>(2*D23*G23)/(2+D23*G23)</f>
+        <v>0.071868393735947</v>
+      </c>
+      <c r="I23" s="55">
+        <f>1-H23</f>
+        <v>0.928131606264053</v>
+      </c>
+      <c r="J23" s="39">
+        <f>J22*I22</f>
+        <v>81679.8400809624</v>
+      </c>
+      <c r="K23" s="39">
+        <f>J23*H23</f>
+        <v>5870.1989072278</v>
+      </c>
+      <c r="L23" s="56" t="n">
         <v>2.5</v>
       </c>
-      <c r="I23" s="55">
-        <f>D23*G23/(1+(D23-H23)*G23)</f>
-        <v>0.071868393735947</v>
-      </c>
-      <c r="J23" s="55">
-        <f>1-I23</f>
-        <v>0.928131606264053</v>
-      </c>
-      <c r="K23" s="39">
-        <f>K22-L22</f>
-        <v>81682.6565813693</v>
-      </c>
-      <c r="L23" s="39">
-        <f>K23*I23</f>
-        <v>5870.40132458799</v>
-      </c>
       <c r="M23" s="39">
-        <f>D23*K24+H23*L23</f>
-        <v>393737.279595376</v>
+        <f>J24*D23+K23*L23</f>
+        <v>393723.703136743</v>
       </c>
       <c r="N23" s="39">
         <f>SUM(M23:$M$25)</f>
-        <v>1871239.74791549</v>
-      </c>
-      <c r="O23" s="56">
-        <f>N23/K23</f>
+        <v>1871175.22568112</v>
+      </c>
+      <c r="O23" s="57">
+        <f>N23/J23</f>
         <v>22.9086543732992</v>
       </c>
       <c r="P23" s="29" t="n"/>
@@ -9351,10 +9298,10 @@
         <f>'Cohorte ficticio'!B63</f>
         <v>70-74</v>
       </c>
-      <c r="C24" s="57" t="n">
+      <c r="C24" s="58" t="n">
         <v>70</v>
       </c>
-      <c r="D24" s="58" t="n">
+      <c r="D24" s="59" t="n">
         <v>5</v>
       </c>
       <c r="E24" s="42">
@@ -9369,36 +9316,35 @@
         <f>F24/E24</f>
         <v>0.0228091266487047</v>
       </c>
-      <c r="H24" s="59">
-        <f>D24/2</f>
+      <c r="H24" s="49">
+        <f>(2*D24*G24)/(2+D24*G24)</f>
+        <v>0.107893255897742</v>
+      </c>
+      <c r="I24" s="49">
+        <f>1-H24</f>
+        <v>0.892106744102258</v>
+      </c>
+      <c r="J24" s="42">
+        <f>J23*I23</f>
+        <v>75809.6411737347</v>
+      </c>
+      <c r="K24" s="42">
+        <f>J24*H24</f>
+        <v>8179.34901467372</v>
+      </c>
+      <c r="L24" s="60" t="n">
         <v>2.5</v>
       </c>
-      <c r="I24" s="49">
-        <f>D24*G24/(1+(D24-H24)*G24)</f>
-        <v>0.107893255897742</v>
-      </c>
-      <c r="J24" s="49">
-        <f>1-I24</f>
-        <v>0.892106744102258</v>
-      </c>
-      <c r="K24" s="42">
-        <f>K23-L23</f>
-        <v>75812.2552567813</v>
-      </c>
-      <c r="L24" s="42">
-        <f>K24*I24</f>
-        <v>8179.63105660481</v>
-      </c>
       <c r="M24" s="42">
-        <f>D24*K25+H24*L24</f>
-        <v>358612.198642394</v>
+        <f>J25*D24+K24*L24</f>
+        <v>358599.833331989</v>
       </c>
       <c r="N24" s="42">
         <f>SUM(M24:$M$25)</f>
-        <v>1477502.46832011</v>
-      </c>
-      <c r="O24" s="60">
-        <f>N24/K24</f>
+        <v>1477451.52254438</v>
+      </c>
+      <c r="O24" s="61">
+        <f>N24/J24</f>
         <v>19.4889660427026</v>
       </c>
       <c r="P24" s="29" t="n"/>
@@ -9429,36 +9375,35 @@
         <f>F25/E25</f>
         <v>0.060446163518481</v>
       </c>
-      <c r="H25" s="61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I25" s="55" t="n">
+      <c r="H25" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="J25" s="55">
-        <f>1-I25</f>
+      <c r="I25" s="55">
+        <f>1-H25</f>
         <v>0</v>
       </c>
+      <c r="J25" s="39">
+        <f>J24*I24</f>
+        <v>67630.2921590609</v>
+      </c>
       <c r="K25" s="39">
-        <f>K24-L24</f>
-        <v>67632.6242001765</v>
-      </c>
-      <c r="L25" s="39">
-        <f>K25*I25</f>
-        <v>67632.6242001765</v>
+        <f>J25*H25</f>
+        <v>67630.2921590609</v>
+      </c>
+      <c r="L25" s="56">
+        <f>1/G25</f>
+        <v>16.5436471364185</v>
       </c>
       <c r="M25" s="39">
-        <f>K25/G25</f>
-        <v>1118890.26967772</v>
+        <f>K25*L25</f>
+        <v>1118851.68921239</v>
       </c>
       <c r="N25" s="39">
         <f>SUM(M25:$M$25)</f>
-        <v>1118890.26967772</v>
-      </c>
-      <c r="O25" s="56">
-        <f>N25/K25</f>
+        <v>1118851.68921239</v>
+      </c>
+      <c r="O25" s="57">
+        <f>N25/J25</f>
         <v>16.5436471364185</v>
       </c>
       <c r="P25" s="29" t="n"/>
@@ -9489,7 +9434,7 @@
         </is>
       </c>
       <c r="E27" s="48">
-        <f>ROUND(SUM(L9:L25)-D5,6)</f>
+        <f>ROUND(SUM(K9:K25)-D5,6)</f>
         <v>0</v>
       </c>
       <c r="F27" s="35" t="inlineStr">
@@ -9510,12 +9455,12 @@
       <c r="A28" s="29" t="n"/>
       <c r="B28" s="62" t="inlineStr">
         <is>
-          <t>q0 (mortalidad infantil, por mil)</t>
-        </is>
-      </c>
-      <c r="E28" s="56">
-        <f>I9*1000</f>
-        <v>8.88817142358165</v>
+          <t>q0 (por mil)</t>
+        </is>
+      </c>
+      <c r="E28" s="57">
+        <f>H9*1000</f>
+        <v>8.92198709250748</v>
       </c>
       <c r="F28" s="29" t="n"/>
       <c r="G28" s="29" t="n"/>
@@ -9810,17 +9755,17 @@
           <t>Esperanza de vida al nacer, e0 (años)</t>
         </is>
       </c>
-      <c r="C7" s="63">
+      <c r="C7" s="56">
         <f>'Tabla hombres'!O9</f>
-        <v>76.6426449219202</v>
-      </c>
-      <c r="D7" s="63">
+        <v>76.6395831777888</v>
+      </c>
+      <c r="D7" s="56">
         <f>'Tabla mujeres'!O9</f>
-        <v>83.9245367809822</v>
-      </c>
-      <c r="E7" s="63">
+        <v>83.9226401604984</v>
+      </c>
+      <c r="E7" s="56">
         <f>'Tabla ambos sexos'!O9</f>
-        <v>80.3094140615</v>
+        <v>80.3069410568805</v>
       </c>
       <c r="F7" s="29" t="n"/>
       <c r="G7" s="29" t="n"/>
@@ -9845,15 +9790,15 @@
           <t>Esperanza de vida a los 5 años, e5</t>
         </is>
       </c>
-      <c r="C8" s="64">
+      <c r="C8" s="60">
         <f>'Tabla hombres'!O11</f>
         <v>72.5564412244842</v>
       </c>
-      <c r="D8" s="64">
+      <c r="D8" s="60">
         <f>'Tabla mujeres'!O11</f>
         <v>79.7255544738942</v>
       </c>
-      <c r="E8" s="64">
+      <c r="E8" s="60">
         <f>'Tabla ambos sexos'!O11</f>
         <v>76.1725915133189</v>
       </c>
@@ -9880,15 +9825,15 @@
           <t>Esperanza de vida a los 65 años, e65</t>
         </is>
       </c>
-      <c r="C9" s="63">
+      <c r="C9" s="56">
         <f>'Tabla hombres'!O22</f>
         <v>24.8083228955963</v>
       </c>
-      <c r="D9" s="63">
+      <c r="D9" s="56">
         <f>'Tabla mujeres'!O22</f>
         <v>28.2448140837104</v>
       </c>
-      <c r="E9" s="63">
+      <c r="E9" s="56">
         <f>'Tabla ambos sexos'!O22</f>
         <v>26.5929390856472</v>
       </c>
@@ -9915,15 +9860,15 @@
           <t>Esperanza de vida a los 75 años, e75</t>
         </is>
       </c>
-      <c r="C10" s="64">
+      <c r="C10" s="60">
         <f>'Tabla hombres'!O25</f>
         <v>15.4605297506321</v>
       </c>
-      <c r="D10" s="64">
+      <c r="D10" s="60">
         <f>'Tabla mujeres'!O25</f>
         <v>17.5038452955524</v>
       </c>
-      <c r="E10" s="64">
+      <c r="E10" s="60">
         <f>'Tabla ambos sexos'!O25</f>
         <v>16.5436471364185</v>
       </c>
@@ -9950,17 +9895,17 @@
           <t>Mortalidad infantil, q0 por mil</t>
         </is>
       </c>
-      <c r="C11" s="63">
-        <f>'Tabla hombres'!I9*1000</f>
-        <v>9.92937335308912</v>
-      </c>
-      <c r="D11" s="63">
-        <f>'Tabla mujeres'!I9*1000</f>
-        <v>7.81956520783196</v>
-      </c>
-      <c r="E11" s="63">
-        <f>'Tabla ambos sexos'!I9*1000</f>
-        <v>8.88817142358165</v>
+      <c r="C11" s="56">
+        <f>'Tabla hombres'!H9*1000</f>
+        <v>9.97176113009477</v>
+      </c>
+      <c r="D11" s="56">
+        <f>'Tabla mujeres'!H9*1000</f>
+        <v>7.84563539639034</v>
+      </c>
+      <c r="E11" s="56">
+        <f>'Tabla ambos sexos'!H9*1000</f>
+        <v>8.92198709250748</v>
       </c>
       <c r="F11" s="29" t="n"/>
       <c r="G11" s="29" t="n"/>
@@ -9985,17 +9930,17 @@
           <t>Mortalidad de menores de 5 años, 5q0 por mil</t>
         </is>
       </c>
-      <c r="C12" s="64">
-        <f>(1-'Tabla hombres'!J9*'Tabla hombres'!J10)*1000</f>
-        <v>11.8567227220026</v>
-      </c>
-      <c r="D12" s="64">
-        <f>(1-'Tabla mujeres'!J9*'Tabla mujeres'!J10)*1000</f>
-        <v>9.51130907831044</v>
-      </c>
-      <c r="E12" s="64">
-        <f>(1-'Tabla ambos sexos'!J9*'Tabla ambos sexos'!J10)*1000</f>
-        <v>10.6991828338718</v>
+      <c r="C12" s="60">
+        <f>(1-'Tabla hombres'!I9*'Tabla hombres'!I10)*1000</f>
+        <v>11.8993818603068</v>
+      </c>
+      <c r="D12" s="60">
+        <f>(1-'Tabla mujeres'!I9*'Tabla mujeres'!I10)*1000</f>
+        <v>9.53768820618029</v>
+      </c>
+      <c r="E12" s="60">
+        <f>(1-'Tabla ambos sexos'!I9*'Tabla ambos sexos'!I10)*1000</f>
+        <v>10.7332949241326</v>
       </c>
       <c r="F12" s="29" t="n"/>
       <c r="G12" s="29" t="n"/>
@@ -10021,16 +9966,16 @@
         </is>
       </c>
       <c r="C13" s="39">
-        <f>'Tabla hombres'!K22</f>
-        <v>81385.29846619</v>
+        <f>'Tabla hombres'!J22</f>
+        <v>81381.784981068</v>
       </c>
       <c r="D13" s="39">
-        <f>'Tabla mujeres'!K22</f>
-        <v>90691.636106611</v>
+        <f>'Tabla mujeres'!J22</f>
+        <v>90689.2207673068</v>
       </c>
       <c r="E13" s="39">
-        <f>'Tabla ambos sexos'!K22</f>
-        <v>86143.346064628</v>
+        <f>'Tabla ambos sexos'!J22</f>
+        <v>86140.3757551475</v>
       </c>
       <c r="F13" s="29" t="n"/>
       <c r="G13" s="29" t="n"/>
@@ -10056,16 +10001,16 @@
         </is>
       </c>
       <c r="C14" s="42">
-        <f>'Tabla hombres'!K25</f>
-        <v>60595.2437917955</v>
+        <f>'Tabla hombres'!J25</f>
+        <v>60592.6278342265</v>
       </c>
       <c r="D14" s="42">
-        <f>'Tabla mujeres'!K25</f>
-        <v>74470.8562173487</v>
+        <f>'Tabla mujeres'!J25</f>
+        <v>74468.8728769464</v>
       </c>
       <c r="E14" s="42">
-        <f>'Tabla ambos sexos'!K25</f>
-        <v>67632.6242001765</v>
+        <f>'Tabla ambos sexos'!J25</f>
+        <v>67630.2921590609</v>
       </c>
       <c r="F14" s="29" t="n"/>
       <c r="G14" s="29" t="n"/>
@@ -10112,13 +10057,13 @@
           <t>e0 de CONAPO, proyecciones 2025 (referencia)</t>
         </is>
       </c>
-      <c r="C16" s="65" t="n">
+      <c r="C16" s="63" t="n">
         <v>72.56999999999999</v>
       </c>
-      <c r="D16" s="65" t="n">
+      <c r="D16" s="63" t="n">
         <v>79.04000000000001</v>
       </c>
-      <c r="E16" s="65" t="n">
+      <c r="E16" s="63" t="n">
         <v>75.67</v>
       </c>
       <c r="F16" s="29" t="n"/>
@@ -10144,17 +10089,17 @@
           <t>Diferencia: estas tablas − CONAPO (años)</t>
         </is>
       </c>
-      <c r="C17" s="64">
+      <c r="C17" s="60">
         <f>C7-C16</f>
-        <v>4.0726449219202</v>
-      </c>
-      <c r="D17" s="64">
+        <v>4.06958317778877</v>
+      </c>
+      <c r="D17" s="60">
         <f>D7-D16</f>
-        <v>4.88453678098223</v>
-      </c>
-      <c r="E17" s="64">
+        <v>4.88264016049843</v>
+      </c>
+      <c r="E17" s="60">
         <f>E7-E16</f>
-        <v>4.63941406149995</v>
+        <v>4.63694105688045</v>
       </c>
       <c r="F17" s="29" t="n"/>
       <c r="G17" s="29" t="n"/>
@@ -10361,7 +10306,7 @@
       <c r="A26" s="29" t="n"/>
       <c r="B26" s="35" t="inlineStr">
         <is>
-          <t>5. nqx = n·nMx / (1 + (n − nax)·nMx), con nax = n/2 salvo 0 y 1-4 (Coale-Demeny). En 75+ se usa e75 = 1/M, muy sensible a las defunciones de adultos mayores.</t>
+          <t>5. nqx = (2·n·nmx) / (2 + n·nmx) y nAx = 0.12, 1.5 y 2.5, como en el ejemplo de la profesora (Cuadro 4.3). En 75+ se usa nAx = 1/nmx, muy sensible a las defunciones de adultos mayores.</t>
         </is>
       </c>
       <c r="F26" s="29" t="n"/>

</xml_diff>